<commit_message>
📊 Actualizar CONSULTA_VENTA_PF.xlsx — 01-04-2026, 3:48:08 p. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_PF.xlsx
+++ b/datos/CONSULTA_VENTA_PF.xlsx
@@ -8,22 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{F0174BB0-E469-4D2D-AB17-F8D404C92624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2DD7123-78EC-4063-B607-B39D1525C7A9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1210F783-412B-4AE0-A961-DAE578DA2515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ParamQuery Pro" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ParamQuery Pro'!$A$1:$AP$101</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4242" uniqueCount="1103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4746" uniqueCount="1213">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -2974,6 +2971,30 @@
     <t>4111</t>
   </si>
   <si>
+    <t>10993874-2</t>
+  </si>
+  <si>
+    <t>RAMIREZ VERA LUIS FREDDY</t>
+  </si>
+  <si>
+    <t>01/05/1969</t>
+  </si>
+  <si>
+    <t>1153 - La Pintana - Santiago -CP</t>
+  </si>
+  <si>
+    <t>950196330</t>
+  </si>
+  <si>
+    <t>ramirezveraveraluis@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>33000</t>
+  </si>
+  <si>
+    <t>4114</t>
+  </si>
+  <si>
     <t>5591009-K</t>
   </si>
   <si>
@@ -3247,6 +3268,42 @@
     <t>4140</t>
   </si>
   <si>
+    <t>20498496-4</t>
+  </si>
+  <si>
+    <t>GUERRERO GODOY BELEN ANDREA</t>
+  </si>
+  <si>
+    <t>01/07/2000</t>
+  </si>
+  <si>
+    <t>5326 - Conchali - Santiago -CP</t>
+  </si>
+  <si>
+    <t>934987237</t>
+  </si>
+  <si>
+    <t>GUERREROGODOYB@GMAIL.COM; ; ; ;</t>
+  </si>
+  <si>
+    <t>1852500</t>
+  </si>
+  <si>
+    <t>1556723</t>
+  </si>
+  <si>
+    <t>185250</t>
+  </si>
+  <si>
+    <t>1667250</t>
+  </si>
+  <si>
+    <t>46313</t>
+  </si>
+  <si>
+    <t>4143</t>
+  </si>
+  <si>
     <t>7420000</t>
   </si>
   <si>
@@ -3265,6 +3322,132 @@
     <t>4146</t>
   </si>
   <si>
+    <t>14130230-2</t>
+  </si>
+  <si>
+    <t>FIGUEROA LUCERO IVETTE LUCIA</t>
+  </si>
+  <si>
+    <t>26/10/1981</t>
+  </si>
+  <si>
+    <t>1183 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>995027541</t>
+  </si>
+  <si>
+    <t>ivt2610@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>ROCIO RAQUEL ALVAREZ SUAREZ</t>
+  </si>
+  <si>
+    <t>3575000</t>
+  </si>
+  <si>
+    <t>3004202</t>
+  </si>
+  <si>
+    <t>357500</t>
+  </si>
+  <si>
+    <t>3217500</t>
+  </si>
+  <si>
+    <t>89375</t>
+  </si>
+  <si>
+    <t>4149</t>
+  </si>
+  <si>
+    <t>10068490-K</t>
+  </si>
+  <si>
+    <t>GAETE OSORIO MARINA DE LAS MERCEDES</t>
+  </si>
+  <si>
+    <t>17/09/1964</t>
+  </si>
+  <si>
+    <t>767 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>988987431</t>
+  </si>
+  <si>
+    <t>marinagaete01@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>160000</t>
+  </si>
+  <si>
+    <t>24407</t>
+  </si>
+  <si>
+    <t>4150</t>
+  </si>
+  <si>
+    <t>16413652-3</t>
+  </si>
+  <si>
+    <t>BRUNA SALAZAR MARIA JOSE</t>
+  </si>
+  <si>
+    <t>20/11/1986</t>
+  </si>
+  <si>
+    <t>744 - San Bernardo - Maipo -CP</t>
+  </si>
+  <si>
+    <t>928835617</t>
+  </si>
+  <si>
+    <t>mariajosebrunasalazar38@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>3600000</t>
+  </si>
+  <si>
+    <t>3025210</t>
+  </si>
+  <si>
+    <t>423000</t>
+  </si>
+  <si>
+    <t>3177000</t>
+  </si>
+  <si>
+    <t>52950</t>
+  </si>
+  <si>
+    <t>4151</t>
+  </si>
+  <si>
+    <t>21706139-3</t>
+  </si>
+  <si>
+    <t>SANCHEZ MARIN MANUELA EXDOSIO</t>
+  </si>
+  <si>
+    <t>15/12/1955</t>
+  </si>
+  <si>
+    <t>3785 - Puente Alto - Cordillera -CP</t>
+  </si>
+  <si>
+    <t>984887271</t>
+  </si>
+  <si>
+    <t>manuela_sanchez55@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>DENISSE XIOMARA MARTÍNEZ TENORIO</t>
+  </si>
+  <si>
+    <t>4152</t>
+  </si>
+  <si>
     <t>9425167-2</t>
   </si>
   <si>
@@ -3292,6 +3475,93 @@
     <t>4154</t>
   </si>
   <si>
+    <t>7899054-6</t>
+  </si>
+  <si>
+    <t>ACUÑA SALAZAR SOLEDAD DEL CARMEN</t>
+  </si>
+  <si>
+    <t>09/01/1957</t>
+  </si>
+  <si>
+    <t>11037 - La Florida - Santiago -CP</t>
+  </si>
+  <si>
+    <t>931082666</t>
+  </si>
+  <si>
+    <t>gonzalomrcl@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>0.54</t>
+  </si>
+  <si>
+    <t>1190000</t>
+  </si>
+  <si>
+    <t>1010000</t>
+  </si>
+  <si>
+    <t>42083</t>
+  </si>
+  <si>
+    <t>4155</t>
+  </si>
+  <si>
+    <t>8346266-3</t>
+  </si>
+  <si>
+    <t>PEÑALOZA PENROZ CRISTIN DEL CARMEN</t>
+  </si>
+  <si>
+    <t>13/01/1958</t>
+  </si>
+  <si>
+    <t>3166 - Puente Alto - Cordillera -CP</t>
+  </si>
+  <si>
+    <t>984656793</t>
+  </si>
+  <si>
+    <t>cristiluna1958@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>39127</t>
+  </si>
+  <si>
+    <t>4161</t>
+  </si>
+  <si>
+    <t>8794589-8</t>
+  </si>
+  <si>
+    <t>SOTO MORALES MARIA ANGELICA</t>
+  </si>
+  <si>
+    <t>15/10/1959</t>
+  </si>
+  <si>
+    <t>2010 - Maipú - Santiago -CP</t>
+  </si>
+  <si>
+    <t>972034665</t>
+  </si>
+  <si>
+    <t>katherinemoralessoto@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>220000</t>
+  </si>
+  <si>
+    <t>1980000</t>
+  </si>
+  <si>
+    <t>55000</t>
+  </si>
+  <si>
+    <t>4163</t>
+  </si>
+  <si>
     <t>8626435-8</t>
   </si>
   <si>
@@ -3310,6 +3580,30 @@
     <t>4165</t>
   </si>
   <si>
+    <t>9128774-9</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ LOPEZ MONICA PATRICIA</t>
+  </si>
+  <si>
+    <t>13/01/1971</t>
+  </si>
+  <si>
+    <t>667 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>975599077</t>
+  </si>
+  <si>
+    <t>mony3203@hotmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>26400</t>
+  </si>
+  <si>
+    <t>4166</t>
+  </si>
+  <si>
     <t>5633286-3</t>
   </si>
   <si>
@@ -3332,6 +3626,39 @@
   </si>
   <si>
     <t>4170</t>
+  </si>
+  <si>
+    <t>4399369-0</t>
+  </si>
+  <si>
+    <t>ALEGRIA HORMAZABAL GERARDO</t>
+  </si>
+  <si>
+    <t>07/09/1940</t>
+  </si>
+  <si>
+    <t>995196937</t>
+  </si>
+  <si>
+    <t>236250</t>
+  </si>
+  <si>
+    <t>4172</t>
+  </si>
+  <si>
+    <t>19570796-0</t>
+  </si>
+  <si>
+    <t>MARTINEZ CONTRERAS RICHARD OMAR</t>
+  </si>
+  <si>
+    <t>25/12/1996</t>
+  </si>
+  <si>
+    <t>937330550</t>
+  </si>
+  <si>
+    <t>4175</t>
   </si>
 </sst>
 </file>
@@ -4192,12 +4519,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP101"/>
+  <dimension ref="A1:AP113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="28" width="8" customWidth="1"/>
-    <col min="29" max="29" width="27.109375" customWidth="1"/>
-    <col min="30" max="41" width="8" customWidth="1"/>
+    <col min="1" max="41" width="8" customWidth="1"/>
     <col min="42" max="42" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -15226,7 +15551,7 @@
         <v>985</v>
       </c>
       <c r="F87" t="s">
-        <v>840</v>
+        <v>736</v>
       </c>
       <c r="G87" t="s">
         <v>986</v>
@@ -15241,7 +15566,7 @@
         <v>988</v>
       </c>
       <c r="K87" t="s">
-        <v>794</v>
+        <v>684</v>
       </c>
       <c r="L87" t="s">
         <v>876</v>
@@ -15253,22 +15578,22 @@
         <v>54</v>
       </c>
       <c r="O87" t="s">
-        <v>398</v>
+        <v>139</v>
       </c>
       <c r="P87" t="s">
-        <v>989</v>
+        <v>577</v>
       </c>
       <c r="Q87" t="s">
-        <v>240</v>
+        <v>142</v>
       </c>
       <c r="R87" t="s">
-        <v>482</v>
+        <v>578</v>
       </c>
       <c r="S87" t="s">
         <v>49</v>
       </c>
       <c r="T87" t="s">
-        <v>511</v>
+        <v>579</v>
       </c>
       <c r="U87" t="s">
         <v>57</v>
@@ -15280,28 +15605,28 @@
         <v>163</v>
       </c>
       <c r="X87" t="s">
-        <v>538</v>
+        <v>580</v>
       </c>
       <c r="Y87" t="s">
         <v>876</v>
       </c>
       <c r="Z87" t="s">
-        <v>350</v>
+        <v>581</v>
       </c>
       <c r="AA87" t="s">
-        <v>342</v>
+        <v>260</v>
       </c>
       <c r="AB87" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="AC87" t="s">
         <v>774</v>
       </c>
       <c r="AD87" t="s">
-        <v>103</v>
+        <v>230</v>
       </c>
       <c r="AE87" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="AF87" t="s">
         <v>65</v>
@@ -15334,7 +15659,7 @@
         <v>49</v>
       </c>
       <c r="AP87" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
     </row>
     <row r="88" spans="1:42" x14ac:dyDescent="0.3">
@@ -15345,31 +15670,31 @@
         <v>43</v>
       </c>
       <c r="C88" t="s">
+        <v>991</v>
+      </c>
+      <c r="D88" t="s">
         <v>992</v>
       </c>
-      <c r="D88" t="s">
+      <c r="E88" t="s">
         <v>993</v>
       </c>
-      <c r="E88" t="s">
+      <c r="F88" t="s">
+        <v>840</v>
+      </c>
+      <c r="G88" t="s">
         <v>994</v>
       </c>
-      <c r="F88" t="s">
+      <c r="H88" t="s">
+        <v>49</v>
+      </c>
+      <c r="I88" t="s">
         <v>995</v>
       </c>
-      <c r="G88" t="s">
+      <c r="J88" t="s">
         <v>996</v>
       </c>
-      <c r="H88" t="s">
-        <v>49</v>
-      </c>
-      <c r="I88" t="s">
-        <v>997</v>
-      </c>
-      <c r="J88" t="s">
-        <v>998</v>
-      </c>
       <c r="K88" t="s">
-        <v>844</v>
+        <v>794</v>
       </c>
       <c r="L88" t="s">
         <v>876</v>
@@ -15381,22 +15706,22 @@
         <v>54</v>
       </c>
       <c r="O88" t="s">
-        <v>55</v>
+        <v>398</v>
       </c>
       <c r="P88" t="s">
-        <v>377</v>
+        <v>997</v>
       </c>
       <c r="Q88" t="s">
-        <v>142</v>
+        <v>240</v>
       </c>
       <c r="R88" t="s">
-        <v>999</v>
+        <v>482</v>
       </c>
       <c r="S88" t="s">
         <v>49</v>
       </c>
       <c r="T88" t="s">
-        <v>1000</v>
+        <v>511</v>
       </c>
       <c r="U88" t="s">
         <v>57</v>
@@ -15408,28 +15733,28 @@
         <v>163</v>
       </c>
       <c r="X88" t="s">
-        <v>1001</v>
+        <v>538</v>
       </c>
       <c r="Y88" t="s">
         <v>876</v>
       </c>
       <c r="Z88" t="s">
-        <v>1002</v>
+        <v>350</v>
       </c>
       <c r="AA88" t="s">
-        <v>178</v>
+        <v>342</v>
       </c>
       <c r="AB88" t="s">
-        <v>1003</v>
+        <v>998</v>
       </c>
       <c r="AC88" t="s">
         <v>774</v>
       </c>
       <c r="AD88" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="AE88" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="AF88" t="s">
         <v>65</v>
@@ -15462,7 +15787,7 @@
         <v>49</v>
       </c>
       <c r="AP88" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
     </row>
     <row r="89" spans="1:42" x14ac:dyDescent="0.3">
@@ -15473,34 +15798,34 @@
         <v>43</v>
       </c>
       <c r="C89" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D89" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E89" t="s">
+        <v>1002</v>
+      </c>
+      <c r="F89" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G89" t="s">
+        <v>1004</v>
+      </c>
+      <c r="H89" t="s">
+        <v>49</v>
+      </c>
+      <c r="I89" t="s">
         <v>1005</v>
       </c>
-      <c r="D89" t="s">
+      <c r="J89" t="s">
         <v>1006</v>
       </c>
-      <c r="E89" t="s">
-        <v>1007</v>
-      </c>
-      <c r="F89" t="s">
-        <v>827</v>
-      </c>
-      <c r="G89" t="s">
-        <v>1008</v>
-      </c>
-      <c r="H89" t="s">
-        <v>1009</v>
-      </c>
-      <c r="I89" t="s">
-        <v>1009</v>
-      </c>
-      <c r="J89" t="s">
-        <v>1010</v>
-      </c>
       <c r="K89" t="s">
-        <v>659</v>
+        <v>844</v>
       </c>
       <c r="L89" t="s">
-        <v>844</v>
+        <v>876</v>
       </c>
       <c r="M89" t="s">
         <v>53</v>
@@ -15509,22 +15834,22 @@
         <v>54</v>
       </c>
       <c r="O89" t="s">
-        <v>139</v>
+        <v>55</v>
       </c>
       <c r="P89" t="s">
-        <v>409</v>
+        <v>377</v>
       </c>
       <c r="Q89" t="s">
-        <v>76</v>
+        <v>142</v>
       </c>
       <c r="R89" t="s">
-        <v>350</v>
+        <v>1007</v>
       </c>
       <c r="S89" t="s">
         <v>49</v>
       </c>
       <c r="T89" t="s">
-        <v>351</v>
+        <v>1008</v>
       </c>
       <c r="U89" t="s">
         <v>57</v>
@@ -15536,16 +15861,16 @@
         <v>163</v>
       </c>
       <c r="X89" t="s">
-        <v>410</v>
+        <v>1009</v>
       </c>
       <c r="Y89" t="s">
-        <v>844</v>
+        <v>876</v>
       </c>
       <c r="Z89" t="s">
-        <v>411</v>
+        <v>1010</v>
       </c>
       <c r="AA89" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="AB89" t="s">
         <v>1011</v>
@@ -15554,10 +15879,10 @@
         <v>774</v>
       </c>
       <c r="AD89" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="AE89" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="AF89" t="s">
         <v>65</v>
@@ -15610,25 +15935,25 @@
         <v>1015</v>
       </c>
       <c r="F90" t="s">
-        <v>995</v>
+        <v>827</v>
       </c>
       <c r="G90" t="s">
-        <v>996</v>
+        <v>1016</v>
       </c>
       <c r="H90" t="s">
-        <v>864</v>
+        <v>1017</v>
       </c>
       <c r="I90" t="s">
-        <v>997</v>
+        <v>1017</v>
       </c>
       <c r="J90" t="s">
-        <v>998</v>
+        <v>1018</v>
       </c>
       <c r="K90" t="s">
+        <v>659</v>
+      </c>
+      <c r="L90" t="s">
         <v>844</v>
-      </c>
-      <c r="L90" t="s">
-        <v>876</v>
       </c>
       <c r="M90" t="s">
         <v>53</v>
@@ -15637,22 +15962,22 @@
         <v>54</v>
       </c>
       <c r="O90" t="s">
-        <v>55</v>
+        <v>139</v>
       </c>
       <c r="P90" t="s">
-        <v>377</v>
+        <v>409</v>
       </c>
       <c r="Q90" t="s">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="R90" t="s">
-        <v>999</v>
+        <v>350</v>
       </c>
       <c r="S90" t="s">
         <v>49</v>
       </c>
       <c r="T90" t="s">
-        <v>1000</v>
+        <v>351</v>
       </c>
       <c r="U90" t="s">
         <v>57</v>
@@ -15664,28 +15989,28 @@
         <v>163</v>
       </c>
       <c r="X90" t="s">
-        <v>1001</v>
+        <v>410</v>
       </c>
       <c r="Y90" t="s">
-        <v>876</v>
+        <v>844</v>
       </c>
       <c r="Z90" t="s">
-        <v>1002</v>
+        <v>411</v>
       </c>
       <c r="AA90" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
       <c r="AB90" t="s">
-        <v>1003</v>
+        <v>1019</v>
       </c>
       <c r="AC90" t="s">
         <v>774</v>
       </c>
       <c r="AD90" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="AE90" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="AF90" t="s">
         <v>65</v>
@@ -15718,7 +16043,7 @@
         <v>49</v>
       </c>
       <c r="AP90" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="91" spans="1:42" x14ac:dyDescent="0.3">
@@ -15729,31 +16054,31 @@
         <v>43</v>
       </c>
       <c r="C91" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="D91" t="s">
-        <v>1018</v>
+        <v>1022</v>
       </c>
       <c r="E91" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
       <c r="F91" t="s">
-        <v>1020</v>
+        <v>1003</v>
       </c>
       <c r="G91" t="s">
-        <v>1021</v>
+        <v>1004</v>
       </c>
       <c r="H91" t="s">
-        <v>49</v>
+        <v>864</v>
       </c>
       <c r="I91" t="s">
-        <v>1022</v>
+        <v>1005</v>
       </c>
       <c r="J91" t="s">
-        <v>1023</v>
+        <v>1006</v>
       </c>
       <c r="K91" t="s">
-        <v>876</v>
+        <v>844</v>
       </c>
       <c r="L91" t="s">
         <v>876</v>
@@ -15765,22 +16090,22 @@
         <v>54</v>
       </c>
       <c r="O91" t="s">
-        <v>590</v>
+        <v>55</v>
       </c>
       <c r="P91" t="s">
-        <v>1024</v>
+        <v>377</v>
       </c>
       <c r="Q91" t="s">
-        <v>211</v>
+        <v>142</v>
       </c>
       <c r="R91" t="s">
-        <v>482</v>
+        <v>1007</v>
       </c>
       <c r="S91" t="s">
         <v>49</v>
       </c>
       <c r="T91" t="s">
-        <v>511</v>
+        <v>1008</v>
       </c>
       <c r="U91" t="s">
         <v>57</v>
@@ -15792,28 +16117,28 @@
         <v>163</v>
       </c>
       <c r="X91" t="s">
-        <v>538</v>
+        <v>1009</v>
       </c>
       <c r="Y91" t="s">
         <v>876</v>
       </c>
       <c r="Z91" t="s">
-        <v>350</v>
+        <v>1010</v>
       </c>
       <c r="AA91" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="AB91" t="s">
-        <v>539</v>
+        <v>1011</v>
       </c>
       <c r="AC91" t="s">
         <v>774</v>
       </c>
       <c r="AD91" t="s">
-        <v>515</v>
+        <v>125</v>
       </c>
       <c r="AE91" t="s">
-        <v>311</v>
+        <v>126</v>
       </c>
       <c r="AF91" t="s">
         <v>65</v>
@@ -15837,7 +16162,7 @@
         <v>49</v>
       </c>
       <c r="AM91" t="s">
-        <v>414</v>
+        <v>66</v>
       </c>
       <c r="AN91" t="s">
         <v>49</v>
@@ -15846,7 +16171,7 @@
         <v>49</v>
       </c>
       <c r="AP91" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="92" spans="1:42" x14ac:dyDescent="0.3">
@@ -15857,16 +16182,16 @@
         <v>43</v>
       </c>
       <c r="C92" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D92" t="s">
         <v>1026</v>
       </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
         <v>1027</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F92" t="s">
         <v>1028</v>
-      </c>
-      <c r="F92" t="s">
-        <v>371</v>
       </c>
       <c r="G92" t="s">
         <v>1029</v>
@@ -15881,7 +16206,7 @@
         <v>1031</v>
       </c>
       <c r="K92" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="L92" t="s">
         <v>876</v>
@@ -15893,7 +16218,7 @@
         <v>54</v>
       </c>
       <c r="O92" t="s">
-        <v>55</v>
+        <v>590</v>
       </c>
       <c r="P92" t="s">
         <v>1032</v>
@@ -15902,13 +16227,13 @@
         <v>211</v>
       </c>
       <c r="R92" t="s">
-        <v>350</v>
+        <v>482</v>
       </c>
       <c r="S92" t="s">
         <v>49</v>
       </c>
       <c r="T92" t="s">
-        <v>351</v>
+        <v>511</v>
       </c>
       <c r="U92" t="s">
         <v>57</v>
@@ -15917,7 +16242,7 @@
         <v>57</v>
       </c>
       <c r="W92" t="s">
-        <v>257</v>
+        <v>163</v>
       </c>
       <c r="X92" t="s">
         <v>538</v>
@@ -15926,22 +16251,22 @@
         <v>876</v>
       </c>
       <c r="Z92" t="s">
-        <v>161</v>
+        <v>350</v>
       </c>
       <c r="AA92" t="s">
-        <v>245</v>
+        <v>148</v>
       </c>
       <c r="AB92" t="s">
-        <v>425</v>
+        <v>539</v>
       </c>
       <c r="AC92" t="s">
         <v>774</v>
       </c>
       <c r="AD92" t="s">
-        <v>110</v>
+        <v>515</v>
       </c>
       <c r="AE92" t="s">
-        <v>111</v>
+        <v>311</v>
       </c>
       <c r="AF92" t="s">
         <v>65</v>
@@ -15965,7 +16290,7 @@
         <v>49</v>
       </c>
       <c r="AM92" t="s">
-        <v>66</v>
+        <v>414</v>
       </c>
       <c r="AN92" t="s">
         <v>49</v>
@@ -15994,13 +16319,13 @@
         <v>1036</v>
       </c>
       <c r="F93" t="s">
-        <v>333</v>
+        <v>371</v>
       </c>
       <c r="G93" t="s">
         <v>1037</v>
       </c>
       <c r="H93" t="s">
-        <v>1038</v>
+        <v>49</v>
       </c>
       <c r="I93" t="s">
         <v>1038</v>
@@ -16009,7 +16334,7 @@
         <v>1039</v>
       </c>
       <c r="K93" t="s">
-        <v>567</v>
+        <v>866</v>
       </c>
       <c r="L93" t="s">
         <v>876</v>
@@ -16021,22 +16346,22 @@
         <v>54</v>
       </c>
       <c r="O93" t="s">
-        <v>338</v>
+        <v>55</v>
       </c>
       <c r="P93" t="s">
-        <v>637</v>
+        <v>1040</v>
       </c>
       <c r="Q93" t="s">
         <v>211</v>
       </c>
       <c r="R93" t="s">
-        <v>897</v>
+        <v>350</v>
       </c>
       <c r="S93" t="s">
         <v>49</v>
       </c>
       <c r="T93" t="s">
-        <v>898</v>
+        <v>351</v>
       </c>
       <c r="U93" t="s">
         <v>57</v>
@@ -16045,31 +16370,31 @@
         <v>57</v>
       </c>
       <c r="W93" t="s">
-        <v>163</v>
+        <v>257</v>
       </c>
       <c r="X93" t="s">
-        <v>1040</v>
+        <v>538</v>
       </c>
       <c r="Y93" t="s">
         <v>876</v>
       </c>
       <c r="Z93" t="s">
-        <v>1041</v>
+        <v>161</v>
       </c>
       <c r="AA93" t="s">
-        <v>184</v>
+        <v>245</v>
       </c>
       <c r="AB93" t="s">
-        <v>1042</v>
+        <v>425</v>
       </c>
       <c r="AC93" t="s">
         <v>774</v>
       </c>
       <c r="AD93" t="s">
-        <v>63</v>
+        <v>110</v>
       </c>
       <c r="AE93" t="s">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="AF93" t="s">
         <v>65</v>
@@ -16102,7 +16427,7 @@
         <v>49</v>
       </c>
       <c r="AP93" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="94" spans="1:42" x14ac:dyDescent="0.3">
@@ -16113,28 +16438,28 @@
         <v>43</v>
       </c>
       <c r="C94" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D94" t="s">
+        <v>1043</v>
+      </c>
+      <c r="E94" t="s">
         <v>1044</v>
-      </c>
-      <c r="D94" t="s">
-        <v>1045</v>
-      </c>
-      <c r="E94" t="s">
-        <v>1046</v>
       </c>
       <c r="F94" t="s">
         <v>333</v>
       </c>
       <c r="G94" t="s">
-        <v>1037</v>
+        <v>1045</v>
       </c>
       <c r="H94" t="s">
+        <v>1046</v>
+      </c>
+      <c r="I94" t="s">
+        <v>1046</v>
+      </c>
+      <c r="J94" t="s">
         <v>1047</v>
-      </c>
-      <c r="I94" t="s">
-        <v>1047</v>
-      </c>
-      <c r="J94" t="s">
-        <v>1048</v>
       </c>
       <c r="K94" t="s">
         <v>567</v>
@@ -16158,13 +16483,13 @@
         <v>211</v>
       </c>
       <c r="R94" t="s">
-        <v>241</v>
+        <v>897</v>
       </c>
       <c r="S94" t="s">
         <v>49</v>
       </c>
       <c r="T94" t="s">
-        <v>242</v>
+        <v>898</v>
       </c>
       <c r="U94" t="s">
         <v>57</v>
@@ -16176,28 +16501,28 @@
         <v>163</v>
       </c>
       <c r="X94" t="s">
-        <v>243</v>
+        <v>1048</v>
       </c>
       <c r="Y94" t="s">
         <v>876</v>
       </c>
       <c r="Z94" t="s">
-        <v>244</v>
+        <v>1049</v>
       </c>
       <c r="AA94" t="s">
-        <v>822</v>
+        <v>184</v>
       </c>
       <c r="AB94" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="AC94" t="s">
         <v>774</v>
       </c>
       <c r="AD94" t="s">
-        <v>125</v>
+        <v>63</v>
       </c>
       <c r="AE94" t="s">
-        <v>126</v>
+        <v>64</v>
       </c>
       <c r="AF94" t="s">
         <v>65</v>
@@ -16230,7 +16555,7 @@
         <v>49</v>
       </c>
       <c r="AP94" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="95" spans="1:42" x14ac:dyDescent="0.3">
@@ -16241,31 +16566,31 @@
         <v>43</v>
       </c>
       <c r="C95" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="D95" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="E95" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="F95" t="s">
-        <v>1054</v>
+        <v>333</v>
       </c>
       <c r="G95" t="s">
+        <v>1045</v>
+      </c>
+      <c r="H95" t="s">
         <v>1055</v>
       </c>
-      <c r="H95" t="s">
+      <c r="I95" t="s">
+        <v>1055</v>
+      </c>
+      <c r="J95" t="s">
         <v>1056</v>
       </c>
-      <c r="I95" t="s">
-        <v>1057</v>
-      </c>
-      <c r="J95" t="s">
-        <v>1058</v>
-      </c>
       <c r="K95" t="s">
-        <v>465</v>
+        <v>567</v>
       </c>
       <c r="L95" t="s">
         <v>876</v>
@@ -16286,13 +16611,13 @@
         <v>211</v>
       </c>
       <c r="R95" t="s">
-        <v>660</v>
+        <v>241</v>
       </c>
       <c r="S95" t="s">
         <v>49</v>
       </c>
       <c r="T95" t="s">
-        <v>661</v>
+        <v>242</v>
       </c>
       <c r="U95" t="s">
         <v>57</v>
@@ -16304,28 +16629,28 @@
         <v>163</v>
       </c>
       <c r="X95" t="s">
-        <v>1059</v>
+        <v>243</v>
       </c>
       <c r="Y95" t="s">
         <v>876</v>
       </c>
       <c r="Z95" t="s">
-        <v>1060</v>
+        <v>244</v>
       </c>
       <c r="AA95" t="s">
-        <v>354</v>
+        <v>822</v>
       </c>
       <c r="AB95" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="AC95" t="s">
         <v>774</v>
       </c>
       <c r="AD95" t="s">
-        <v>262</v>
+        <v>125</v>
       </c>
       <c r="AE95" t="s">
-        <v>263</v>
+        <v>126</v>
       </c>
       <c r="AF95" t="s">
         <v>65</v>
@@ -16358,7 +16683,7 @@
         <v>49</v>
       </c>
       <c r="AP95" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="96" spans="1:42" x14ac:dyDescent="0.3">
@@ -16369,34 +16694,34 @@
         <v>43</v>
       </c>
       <c r="C96" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D96" t="s">
+        <v>1060</v>
+      </c>
+      <c r="E96" t="s">
+        <v>1061</v>
+      </c>
+      <c r="F96" t="s">
+        <v>1062</v>
+      </c>
+      <c r="G96" t="s">
         <v>1063</v>
       </c>
-      <c r="D96" t="s">
+      <c r="H96" t="s">
         <v>1064</v>
       </c>
-      <c r="E96" t="s">
+      <c r="I96" t="s">
         <v>1065</v>
       </c>
-      <c r="F96" t="s">
-        <v>235</v>
-      </c>
-      <c r="G96" t="s">
+      <c r="J96" t="s">
         <v>1066</v>
       </c>
-      <c r="H96" t="s">
-        <v>49</v>
-      </c>
-      <c r="I96" t="s">
-        <v>1067</v>
-      </c>
-      <c r="J96" t="s">
-        <v>1068</v>
-      </c>
       <c r="K96" t="s">
-        <v>844</v>
+        <v>465</v>
       </c>
       <c r="L96" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="M96" t="s">
         <v>53</v>
@@ -16405,22 +16730,22 @@
         <v>54</v>
       </c>
       <c r="O96" t="s">
-        <v>398</v>
+        <v>338</v>
       </c>
       <c r="P96" t="s">
-        <v>1069</v>
+        <v>637</v>
       </c>
       <c r="Q96" t="s">
         <v>211</v>
       </c>
       <c r="R96" t="s">
-        <v>58</v>
+        <v>660</v>
       </c>
       <c r="S96" t="s">
         <v>49</v>
       </c>
       <c r="T96" t="s">
-        <v>59</v>
+        <v>661</v>
       </c>
       <c r="U96" t="s">
         <v>57</v>
@@ -16432,28 +16757,28 @@
         <v>163</v>
       </c>
       <c r="X96" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="Y96" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="Z96" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="AA96" t="s">
-        <v>95</v>
+        <v>354</v>
       </c>
       <c r="AB96" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
       <c r="AC96" t="s">
         <v>774</v>
       </c>
       <c r="AD96" t="s">
-        <v>952</v>
+        <v>262</v>
       </c>
       <c r="AE96" t="s">
-        <v>126</v>
+        <v>263</v>
       </c>
       <c r="AF96" t="s">
         <v>65</v>
@@ -16486,7 +16811,7 @@
         <v>49</v>
       </c>
       <c r="AP96" t="s">
-        <v>1073</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="97" spans="1:42" x14ac:dyDescent="0.3">
@@ -16497,34 +16822,34 @@
         <v>43</v>
       </c>
       <c r="C97" t="s">
-        <v>905</v>
+        <v>1071</v>
       </c>
       <c r="D97" t="s">
-        <v>906</v>
+        <v>1072</v>
       </c>
       <c r="E97" t="s">
-        <v>907</v>
+        <v>1073</v>
       </c>
       <c r="F97" t="s">
-        <v>89</v>
+        <v>235</v>
       </c>
       <c r="G97" t="s">
-        <v>908</v>
+        <v>1074</v>
       </c>
       <c r="H97" t="s">
-        <v>909</v>
+        <v>49</v>
       </c>
       <c r="I97" t="s">
-        <v>909</v>
+        <v>1075</v>
       </c>
       <c r="J97" t="s">
-        <v>910</v>
+        <v>1076</v>
       </c>
       <c r="K97" t="s">
-        <v>876</v>
+        <v>844</v>
       </c>
       <c r="L97" t="s">
-        <v>876</v>
+        <v>866</v>
       </c>
       <c r="M97" t="s">
         <v>53</v>
@@ -16536,19 +16861,19 @@
         <v>398</v>
       </c>
       <c r="P97" t="s">
-        <v>399</v>
+        <v>1077</v>
       </c>
       <c r="Q97" t="s">
-        <v>626</v>
+        <v>211</v>
       </c>
       <c r="R97" t="s">
-        <v>1074</v>
+        <v>58</v>
       </c>
       <c r="S97" t="s">
         <v>49</v>
       </c>
       <c r="T97" t="s">
-        <v>1075</v>
+        <v>59</v>
       </c>
       <c r="U97" t="s">
         <v>57</v>
@@ -16560,28 +16885,28 @@
         <v>163</v>
       </c>
       <c r="X97" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="Y97" t="s">
-        <v>876</v>
+        <v>866</v>
       </c>
       <c r="Z97" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="AA97" t="s">
-        <v>148</v>
+        <v>95</v>
       </c>
       <c r="AB97" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="AC97" t="s">
         <v>774</v>
       </c>
       <c r="AD97" t="s">
-        <v>150</v>
+        <v>952</v>
       </c>
       <c r="AE97" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
       <c r="AF97" t="s">
         <v>65</v>
@@ -16614,7 +16939,7 @@
         <v>49</v>
       </c>
       <c r="AP97" t="s">
-        <v>1079</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="98" spans="1:42" x14ac:dyDescent="0.3">
@@ -16625,31 +16950,31 @@
         <v>43</v>
       </c>
       <c r="C98" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="D98" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="E98" t="s">
-        <v>1082</v>
+        <v>1084</v>
       </c>
       <c r="F98" t="s">
-        <v>995</v>
+        <v>251</v>
       </c>
       <c r="G98" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="H98" t="s">
         <v>49</v>
       </c>
       <c r="I98" t="s">
-        <v>1084</v>
+        <v>1086</v>
       </c>
       <c r="J98" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="K98" t="s">
-        <v>866</v>
+        <v>844</v>
       </c>
       <c r="L98" t="s">
         <v>866</v>
@@ -16661,22 +16986,22 @@
         <v>54</v>
       </c>
       <c r="O98" t="s">
-        <v>398</v>
+        <v>139</v>
       </c>
       <c r="P98" t="s">
-        <v>1086</v>
+        <v>449</v>
       </c>
       <c r="Q98" t="s">
-        <v>57</v>
+        <v>211</v>
       </c>
       <c r="R98" t="s">
-        <v>122</v>
+        <v>1088</v>
       </c>
       <c r="S98" t="s">
         <v>49</v>
       </c>
       <c r="T98" t="s">
-        <v>123</v>
+        <v>1089</v>
       </c>
       <c r="U98" t="s">
         <v>57</v>
@@ -16685,22 +17010,22 @@
         <v>57</v>
       </c>
       <c r="W98" t="s">
-        <v>60</v>
+        <v>163</v>
       </c>
       <c r="X98" t="s">
-        <v>122</v>
+        <v>1090</v>
       </c>
       <c r="Y98" t="s">
         <v>866</v>
       </c>
       <c r="Z98" t="s">
-        <v>49</v>
+        <v>1091</v>
       </c>
       <c r="AA98" t="s">
-        <v>857</v>
+        <v>148</v>
       </c>
       <c r="AB98" t="s">
-        <v>122</v>
+        <v>1092</v>
       </c>
       <c r="AC98" t="s">
         <v>774</v>
@@ -16742,7 +17067,7 @@
         <v>49</v>
       </c>
       <c r="AP98" t="s">
-        <v>1087</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="99" spans="1:42" x14ac:dyDescent="0.3">
@@ -16753,34 +17078,34 @@
         <v>43</v>
       </c>
       <c r="C99" t="s">
-        <v>1080</v>
+        <v>905</v>
       </c>
       <c r="D99" t="s">
-        <v>1081</v>
+        <v>906</v>
       </c>
       <c r="E99" t="s">
-        <v>1082</v>
+        <v>907</v>
       </c>
       <c r="F99" t="s">
-        <v>995</v>
+        <v>89</v>
       </c>
       <c r="G99" t="s">
-        <v>1083</v>
+        <v>908</v>
       </c>
       <c r="H99" t="s">
-        <v>49</v>
+        <v>909</v>
       </c>
       <c r="I99" t="s">
-        <v>1084</v>
+        <v>909</v>
       </c>
       <c r="J99" t="s">
-        <v>1085</v>
+        <v>910</v>
       </c>
       <c r="K99" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="L99" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="M99" t="s">
         <v>53</v>
@@ -16792,19 +17117,19 @@
         <v>398</v>
       </c>
       <c r="P99" t="s">
-        <v>1086</v>
+        <v>399</v>
       </c>
       <c r="Q99" t="s">
-        <v>57</v>
+        <v>626</v>
       </c>
       <c r="R99" t="s">
-        <v>122</v>
+        <v>1094</v>
       </c>
       <c r="S99" t="s">
         <v>49</v>
       </c>
       <c r="T99" t="s">
-        <v>123</v>
+        <v>1095</v>
       </c>
       <c r="U99" t="s">
         <v>57</v>
@@ -16813,31 +17138,31 @@
         <v>57</v>
       </c>
       <c r="W99" t="s">
-        <v>60</v>
+        <v>163</v>
       </c>
       <c r="X99" t="s">
-        <v>122</v>
+        <v>1096</v>
       </c>
       <c r="Y99" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="Z99" t="s">
-        <v>49</v>
+        <v>1097</v>
       </c>
       <c r="AA99" t="s">
-        <v>857</v>
+        <v>148</v>
       </c>
       <c r="AB99" t="s">
-        <v>122</v>
+        <v>1098</v>
       </c>
       <c r="AC99" t="s">
         <v>774</v>
       </c>
       <c r="AD99" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="AE99" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="AF99" t="s">
         <v>65</v>
@@ -16870,7 +17195,7 @@
         <v>49</v>
       </c>
       <c r="AP99" t="s">
-        <v>1088</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="100" spans="1:42" x14ac:dyDescent="0.3">
@@ -16881,34 +17206,34 @@
         <v>43</v>
       </c>
       <c r="C100" t="s">
-        <v>1089</v>
+        <v>1100</v>
       </c>
       <c r="D100" t="s">
-        <v>1090</v>
+        <v>1101</v>
       </c>
       <c r="E100" t="s">
-        <v>1091</v>
+        <v>1102</v>
       </c>
       <c r="F100" t="s">
-        <v>827</v>
+        <v>156</v>
       </c>
       <c r="G100" t="s">
-        <v>1008</v>
+        <v>1103</v>
       </c>
       <c r="H100" t="s">
-        <v>1092</v>
+        <v>49</v>
       </c>
       <c r="I100" t="s">
-        <v>1009</v>
+        <v>1104</v>
       </c>
       <c r="J100" t="s">
-        <v>1010</v>
+        <v>1105</v>
       </c>
       <c r="K100" t="s">
-        <v>659</v>
+        <v>866</v>
       </c>
       <c r="L100" t="s">
-        <v>876</v>
+        <v>866</v>
       </c>
       <c r="M100" t="s">
         <v>53</v>
@@ -16920,19 +17245,19 @@
         <v>139</v>
       </c>
       <c r="P100" t="s">
-        <v>1093</v>
+        <v>1106</v>
       </c>
       <c r="Q100" t="s">
-        <v>76</v>
+        <v>211</v>
       </c>
       <c r="R100" t="s">
-        <v>350</v>
+        <v>1107</v>
       </c>
       <c r="S100" t="s">
         <v>49</v>
       </c>
       <c r="T100" t="s">
-        <v>351</v>
+        <v>1108</v>
       </c>
       <c r="U100" t="s">
         <v>57</v>
@@ -16944,28 +17269,28 @@
         <v>163</v>
       </c>
       <c r="X100" t="s">
-        <v>410</v>
+        <v>1109</v>
       </c>
       <c r="Y100" t="s">
-        <v>876</v>
+        <v>866</v>
       </c>
       <c r="Z100" t="s">
-        <v>411</v>
+        <v>1110</v>
       </c>
       <c r="AA100" t="s">
         <v>148</v>
       </c>
       <c r="AB100" t="s">
-        <v>1011</v>
+        <v>1111</v>
       </c>
       <c r="AC100" t="s">
         <v>774</v>
       </c>
       <c r="AD100" t="s">
-        <v>110</v>
+        <v>455</v>
       </c>
       <c r="AE100" t="s">
-        <v>111</v>
+        <v>456</v>
       </c>
       <c r="AF100" t="s">
         <v>65</v>
@@ -16998,7 +17323,7 @@
         <v>49</v>
       </c>
       <c r="AP100" t="s">
-        <v>1094</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="101" spans="1:42" x14ac:dyDescent="0.3">
@@ -17009,34 +17334,34 @@
         <v>43</v>
       </c>
       <c r="C101" t="s">
-        <v>1095</v>
+        <v>1113</v>
       </c>
       <c r="D101" t="s">
-        <v>1096</v>
+        <v>1114</v>
       </c>
       <c r="E101" t="s">
-        <v>1097</v>
+        <v>1115</v>
       </c>
       <c r="F101" t="s">
-        <v>235</v>
+        <v>156</v>
       </c>
       <c r="G101" t="s">
-        <v>1098</v>
+        <v>1116</v>
       </c>
       <c r="H101" t="s">
-        <v>49</v>
+        <v>1117</v>
       </c>
       <c r="I101" t="s">
-        <v>1099</v>
+        <v>1117</v>
       </c>
       <c r="J101" t="s">
-        <v>1100</v>
+        <v>1118</v>
       </c>
       <c r="K101" t="s">
+        <v>844</v>
+      </c>
+      <c r="L101" t="s">
         <v>866</v>
-      </c>
-      <c r="L101" t="s">
-        <v>876</v>
       </c>
       <c r="M101" t="s">
         <v>53</v>
@@ -17045,22 +17370,22 @@
         <v>54</v>
       </c>
       <c r="O101" t="s">
-        <v>139</v>
+        <v>398</v>
       </c>
       <c r="P101" t="s">
-        <v>439</v>
+        <v>399</v>
       </c>
       <c r="Q101" t="s">
-        <v>95</v>
+        <v>626</v>
       </c>
       <c r="R101" t="s">
-        <v>897</v>
+        <v>512</v>
       </c>
       <c r="S101" t="s">
         <v>49</v>
       </c>
       <c r="T101" t="s">
-        <v>898</v>
+        <v>741</v>
       </c>
       <c r="U101" t="s">
         <v>57</v>
@@ -17072,28 +17397,28 @@
         <v>163</v>
       </c>
       <c r="X101" t="s">
-        <v>1040</v>
+        <v>1119</v>
       </c>
       <c r="Y101" t="s">
-        <v>876</v>
+        <v>866</v>
       </c>
       <c r="Z101" t="s">
-        <v>1041</v>
+        <v>161</v>
       </c>
       <c r="AA101" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="AB101" t="s">
-        <v>1101</v>
+        <v>1120</v>
       </c>
       <c r="AC101" t="s">
         <v>774</v>
       </c>
       <c r="AD101" t="s">
-        <v>63</v>
+        <v>515</v>
       </c>
       <c r="AE101" t="s">
-        <v>64</v>
+        <v>311</v>
       </c>
       <c r="AF101" t="s">
         <v>65</v>
@@ -17126,11 +17451,1546 @@
         <v>49</v>
       </c>
       <c r="AP101" t="s">
-        <v>1102</v>
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="102" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>42</v>
+      </c>
+      <c r="B102" t="s">
+        <v>43</v>
+      </c>
+      <c r="C102" t="s">
+        <v>1122</v>
+      </c>
+      <c r="D102" t="s">
+        <v>1123</v>
+      </c>
+      <c r="E102" t="s">
+        <v>1124</v>
+      </c>
+      <c r="F102" t="s">
+        <v>371</v>
+      </c>
+      <c r="G102" t="s">
+        <v>1125</v>
+      </c>
+      <c r="H102" t="s">
+        <v>1126</v>
+      </c>
+      <c r="I102" t="s">
+        <v>1126</v>
+      </c>
+      <c r="J102" t="s">
+        <v>1127</v>
+      </c>
+      <c r="K102" t="s">
+        <v>817</v>
+      </c>
+      <c r="L102" t="s">
+        <v>876</v>
+      </c>
+      <c r="M102" t="s">
+        <v>53</v>
+      </c>
+      <c r="N102" t="s">
+        <v>54</v>
+      </c>
+      <c r="O102" t="s">
+        <v>854</v>
+      </c>
+      <c r="P102" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q102" t="s">
+        <v>76</v>
+      </c>
+      <c r="R102" t="s">
+        <v>1128</v>
+      </c>
+      <c r="S102" t="s">
+        <v>49</v>
+      </c>
+      <c r="T102" t="s">
+        <v>1129</v>
+      </c>
+      <c r="U102" t="s">
+        <v>57</v>
+      </c>
+      <c r="V102" t="s">
+        <v>57</v>
+      </c>
+      <c r="W102" t="s">
+        <v>79</v>
+      </c>
+      <c r="X102" t="s">
+        <v>1130</v>
+      </c>
+      <c r="Y102" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z102" t="s">
+        <v>1131</v>
+      </c>
+      <c r="AA102" t="s">
+        <v>226</v>
+      </c>
+      <c r="AB102" t="s">
+        <v>1132</v>
+      </c>
+      <c r="AC102" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD102" t="s">
+        <v>967</v>
+      </c>
+      <c r="AE102" t="s">
+        <v>456</v>
+      </c>
+      <c r="AF102" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG102" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH102" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI102" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ102" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK102" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL102" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM102" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN102" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO102" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP102" t="s">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="103" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>42</v>
+      </c>
+      <c r="B103" t="s">
+        <v>43</v>
+      </c>
+      <c r="C103" t="s">
+        <v>1134</v>
+      </c>
+      <c r="D103" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E103" t="s">
+        <v>1136</v>
+      </c>
+      <c r="F103" t="s">
+        <v>89</v>
+      </c>
+      <c r="G103" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H103" t="s">
+        <v>49</v>
+      </c>
+      <c r="I103" t="s">
+        <v>1138</v>
+      </c>
+      <c r="J103" t="s">
+        <v>1139</v>
+      </c>
+      <c r="K103" t="s">
+        <v>866</v>
+      </c>
+      <c r="L103" t="s">
+        <v>866</v>
+      </c>
+      <c r="M103" t="s">
+        <v>53</v>
+      </c>
+      <c r="N103" t="s">
+        <v>54</v>
+      </c>
+      <c r="O103" t="s">
+        <v>961</v>
+      </c>
+      <c r="P103" t="s">
+        <v>1140</v>
+      </c>
+      <c r="Q103" t="s">
+        <v>211</v>
+      </c>
+      <c r="R103" t="s">
+        <v>482</v>
+      </c>
+      <c r="S103" t="s">
+        <v>49</v>
+      </c>
+      <c r="T103" t="s">
+        <v>511</v>
+      </c>
+      <c r="U103" t="s">
+        <v>57</v>
+      </c>
+      <c r="V103" t="s">
+        <v>57</v>
+      </c>
+      <c r="W103" t="s">
+        <v>163</v>
+      </c>
+      <c r="X103" t="s">
+        <v>538</v>
+      </c>
+      <c r="Y103" t="s">
+        <v>866</v>
+      </c>
+      <c r="Z103" t="s">
+        <v>350</v>
+      </c>
+      <c r="AA103" t="s">
+        <v>412</v>
+      </c>
+      <c r="AB103" t="s">
+        <v>539</v>
+      </c>
+      <c r="AC103" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD103" t="s">
+        <v>103</v>
+      </c>
+      <c r="AE103" t="s">
+        <v>84</v>
+      </c>
+      <c r="AF103" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG103" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH103" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI103" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ103" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK103" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL103" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM103" t="s">
+        <v>414</v>
+      </c>
+      <c r="AN103" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO103" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP103" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="104" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>42</v>
+      </c>
+      <c r="B104" t="s">
+        <v>43</v>
+      </c>
+      <c r="C104" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D104" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E104" t="s">
+        <v>1144</v>
+      </c>
+      <c r="F104" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G104" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H104" t="s">
+        <v>49</v>
+      </c>
+      <c r="I104" t="s">
+        <v>1146</v>
+      </c>
+      <c r="J104" t="s">
+        <v>1147</v>
+      </c>
+      <c r="K104" t="s">
+        <v>866</v>
+      </c>
+      <c r="L104" t="s">
+        <v>866</v>
+      </c>
+      <c r="M104" t="s">
+        <v>53</v>
+      </c>
+      <c r="N104" t="s">
+        <v>54</v>
+      </c>
+      <c r="O104" t="s">
+        <v>398</v>
+      </c>
+      <c r="P104" t="s">
+        <v>1148</v>
+      </c>
+      <c r="Q104" t="s">
+        <v>57</v>
+      </c>
+      <c r="R104" t="s">
+        <v>122</v>
+      </c>
+      <c r="S104" t="s">
+        <v>49</v>
+      </c>
+      <c r="T104" t="s">
+        <v>123</v>
+      </c>
+      <c r="U104" t="s">
+        <v>57</v>
+      </c>
+      <c r="V104" t="s">
+        <v>57</v>
+      </c>
+      <c r="W104" t="s">
+        <v>60</v>
+      </c>
+      <c r="X104" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y104" t="s">
+        <v>866</v>
+      </c>
+      <c r="Z104" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA104" t="s">
+        <v>857</v>
+      </c>
+      <c r="AB104" t="s">
+        <v>122</v>
+      </c>
+      <c r="AC104" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD104" t="s">
+        <v>125</v>
+      </c>
+      <c r="AE104" t="s">
+        <v>126</v>
+      </c>
+      <c r="AF104" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG104" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH104" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI104" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ104" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK104" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL104" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM104" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN104" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO104" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP104" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="105" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>42</v>
+      </c>
+      <c r="B105" t="s">
+        <v>43</v>
+      </c>
+      <c r="C105" t="s">
+        <v>1142</v>
+      </c>
+      <c r="D105" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E105" t="s">
+        <v>1144</v>
+      </c>
+      <c r="F105" t="s">
+        <v>1003</v>
+      </c>
+      <c r="G105" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H105" t="s">
+        <v>49</v>
+      </c>
+      <c r="I105" t="s">
+        <v>1146</v>
+      </c>
+      <c r="J105" t="s">
+        <v>1147</v>
+      </c>
+      <c r="K105" t="s">
+        <v>866</v>
+      </c>
+      <c r="L105" t="s">
+        <v>866</v>
+      </c>
+      <c r="M105" t="s">
+        <v>53</v>
+      </c>
+      <c r="N105" t="s">
+        <v>54</v>
+      </c>
+      <c r="O105" t="s">
+        <v>398</v>
+      </c>
+      <c r="P105" t="s">
+        <v>1148</v>
+      </c>
+      <c r="Q105" t="s">
+        <v>57</v>
+      </c>
+      <c r="R105" t="s">
+        <v>122</v>
+      </c>
+      <c r="S105" t="s">
+        <v>49</v>
+      </c>
+      <c r="T105" t="s">
+        <v>123</v>
+      </c>
+      <c r="U105" t="s">
+        <v>57</v>
+      </c>
+      <c r="V105" t="s">
+        <v>57</v>
+      </c>
+      <c r="W105" t="s">
+        <v>60</v>
+      </c>
+      <c r="X105" t="s">
+        <v>122</v>
+      </c>
+      <c r="Y105" t="s">
+        <v>866</v>
+      </c>
+      <c r="Z105" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA105" t="s">
+        <v>857</v>
+      </c>
+      <c r="AB105" t="s">
+        <v>122</v>
+      </c>
+      <c r="AC105" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD105" t="s">
+        <v>125</v>
+      </c>
+      <c r="AE105" t="s">
+        <v>126</v>
+      </c>
+      <c r="AF105" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG105" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH105" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI105" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ105" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK105" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL105" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM105" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN105" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO105" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP105" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="106" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>42</v>
+      </c>
+      <c r="B106" t="s">
+        <v>43</v>
+      </c>
+      <c r="C106" t="s">
+        <v>1151</v>
+      </c>
+      <c r="D106" t="s">
+        <v>1152</v>
+      </c>
+      <c r="E106" t="s">
+        <v>1153</v>
+      </c>
+      <c r="F106" t="s">
+        <v>172</v>
+      </c>
+      <c r="G106" t="s">
+        <v>1154</v>
+      </c>
+      <c r="H106" t="s">
+        <v>49</v>
+      </c>
+      <c r="I106" t="s">
+        <v>1155</v>
+      </c>
+      <c r="J106" t="s">
+        <v>1156</v>
+      </c>
+      <c r="K106" t="s">
+        <v>866</v>
+      </c>
+      <c r="L106" t="s">
+        <v>876</v>
+      </c>
+      <c r="M106" t="s">
+        <v>53</v>
+      </c>
+      <c r="N106" t="s">
+        <v>54</v>
+      </c>
+      <c r="O106" t="s">
+        <v>398</v>
+      </c>
+      <c r="P106" t="s">
+        <v>625</v>
+      </c>
+      <c r="Q106" t="s">
+        <v>240</v>
+      </c>
+      <c r="R106" t="s">
+        <v>183</v>
+      </c>
+      <c r="S106" t="s">
+        <v>49</v>
+      </c>
+      <c r="T106" t="s">
+        <v>466</v>
+      </c>
+      <c r="U106" t="s">
+        <v>57</v>
+      </c>
+      <c r="V106" t="s">
+        <v>57</v>
+      </c>
+      <c r="W106" t="s">
+        <v>1157</v>
+      </c>
+      <c r="X106" t="s">
+        <v>1158</v>
+      </c>
+      <c r="Y106" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z106" t="s">
+        <v>1159</v>
+      </c>
+      <c r="AA106" t="s">
+        <v>569</v>
+      </c>
+      <c r="AB106" t="s">
+        <v>1160</v>
+      </c>
+      <c r="AC106" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD106" t="s">
+        <v>230</v>
+      </c>
+      <c r="AE106" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF106" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG106" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH106" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI106" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ106" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK106" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL106" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM106" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN106" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO106" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP106" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="107" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>42</v>
+      </c>
+      <c r="B107" t="s">
+        <v>43</v>
+      </c>
+      <c r="C107" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D107" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E107" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F107" t="s">
+        <v>89</v>
+      </c>
+      <c r="G107" t="s">
+        <v>1165</v>
+      </c>
+      <c r="H107" t="s">
+        <v>49</v>
+      </c>
+      <c r="I107" t="s">
+        <v>1166</v>
+      </c>
+      <c r="J107" t="s">
+        <v>1167</v>
+      </c>
+      <c r="K107" t="s">
+        <v>684</v>
+      </c>
+      <c r="L107" t="s">
+        <v>876</v>
+      </c>
+      <c r="M107" t="s">
+        <v>53</v>
+      </c>
+      <c r="N107" t="s">
+        <v>54</v>
+      </c>
+      <c r="O107" t="s">
+        <v>398</v>
+      </c>
+      <c r="P107" t="s">
+        <v>685</v>
+      </c>
+      <c r="Q107" t="s">
+        <v>626</v>
+      </c>
+      <c r="R107" t="s">
+        <v>241</v>
+      </c>
+      <c r="S107" t="s">
+        <v>49</v>
+      </c>
+      <c r="T107" t="s">
+        <v>242</v>
+      </c>
+      <c r="U107" t="s">
+        <v>57</v>
+      </c>
+      <c r="V107" t="s">
+        <v>57</v>
+      </c>
+      <c r="W107" t="s">
+        <v>163</v>
+      </c>
+      <c r="X107" t="s">
+        <v>243</v>
+      </c>
+      <c r="Y107" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z107" t="s">
+        <v>244</v>
+      </c>
+      <c r="AA107" t="s">
+        <v>178</v>
+      </c>
+      <c r="AB107" t="s">
+        <v>1168</v>
+      </c>
+      <c r="AC107" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD107" t="s">
+        <v>125</v>
+      </c>
+      <c r="AE107" t="s">
+        <v>126</v>
+      </c>
+      <c r="AF107" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG107" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH107" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI107" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ107" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK107" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL107" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM107" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN107" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO107" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP107" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="108" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>42</v>
+      </c>
+      <c r="B108" t="s">
+        <v>43</v>
+      </c>
+      <c r="C108" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D108" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E108" t="s">
+        <v>1172</v>
+      </c>
+      <c r="F108" t="s">
+        <v>235</v>
+      </c>
+      <c r="G108" t="s">
+        <v>1173</v>
+      </c>
+      <c r="H108" t="s">
+        <v>49</v>
+      </c>
+      <c r="I108" t="s">
+        <v>1174</v>
+      </c>
+      <c r="J108" t="s">
+        <v>1175</v>
+      </c>
+      <c r="K108" t="s">
+        <v>876</v>
+      </c>
+      <c r="L108" t="s">
+        <v>876</v>
+      </c>
+      <c r="M108" t="s">
+        <v>53</v>
+      </c>
+      <c r="N108" t="s">
+        <v>54</v>
+      </c>
+      <c r="O108" t="s">
+        <v>338</v>
+      </c>
+      <c r="P108" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q108" t="s">
+        <v>211</v>
+      </c>
+      <c r="R108" t="s">
+        <v>183</v>
+      </c>
+      <c r="S108" t="s">
+        <v>49</v>
+      </c>
+      <c r="T108" t="s">
+        <v>466</v>
+      </c>
+      <c r="U108" t="s">
+        <v>57</v>
+      </c>
+      <c r="V108" t="s">
+        <v>57</v>
+      </c>
+      <c r="W108" t="s">
+        <v>163</v>
+      </c>
+      <c r="X108" t="s">
+        <v>1176</v>
+      </c>
+      <c r="Y108" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z108" t="s">
+        <v>1177</v>
+      </c>
+      <c r="AA108" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB108" t="s">
+        <v>1178</v>
+      </c>
+      <c r="AC108" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD108" t="s">
+        <v>230</v>
+      </c>
+      <c r="AE108" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF108" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG108" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH108" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI108" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ108" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK108" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL108" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM108" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN108" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO108" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP108" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="109" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>42</v>
+      </c>
+      <c r="B109" t="s">
+        <v>43</v>
+      </c>
+      <c r="C109" t="s">
+        <v>1180</v>
+      </c>
+      <c r="D109" t="s">
+        <v>1181</v>
+      </c>
+      <c r="E109" t="s">
+        <v>1182</v>
+      </c>
+      <c r="F109" t="s">
+        <v>827</v>
+      </c>
+      <c r="G109" t="s">
+        <v>1016</v>
+      </c>
+      <c r="H109" t="s">
+        <v>1183</v>
+      </c>
+      <c r="I109" t="s">
+        <v>1017</v>
+      </c>
+      <c r="J109" t="s">
+        <v>1018</v>
+      </c>
+      <c r="K109" t="s">
+        <v>659</v>
+      </c>
+      <c r="L109" t="s">
+        <v>876</v>
+      </c>
+      <c r="M109" t="s">
+        <v>53</v>
+      </c>
+      <c r="N109" t="s">
+        <v>54</v>
+      </c>
+      <c r="O109" t="s">
+        <v>139</v>
+      </c>
+      <c r="P109" t="s">
+        <v>1184</v>
+      </c>
+      <c r="Q109" t="s">
+        <v>76</v>
+      </c>
+      <c r="R109" t="s">
+        <v>350</v>
+      </c>
+      <c r="S109" t="s">
+        <v>49</v>
+      </c>
+      <c r="T109" t="s">
+        <v>351</v>
+      </c>
+      <c r="U109" t="s">
+        <v>57</v>
+      </c>
+      <c r="V109" t="s">
+        <v>57</v>
+      </c>
+      <c r="W109" t="s">
+        <v>163</v>
+      </c>
+      <c r="X109" t="s">
+        <v>410</v>
+      </c>
+      <c r="Y109" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z109" t="s">
+        <v>411</v>
+      </c>
+      <c r="AA109" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB109" t="s">
+        <v>1019</v>
+      </c>
+      <c r="AC109" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD109" t="s">
+        <v>110</v>
+      </c>
+      <c r="AE109" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF109" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG109" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH109" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI109" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ109" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK109" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL109" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM109" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN109" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO109" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP109" t="s">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="110" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>42</v>
+      </c>
+      <c r="B110" t="s">
+        <v>43</v>
+      </c>
+      <c r="C110" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D110" t="s">
+        <v>1187</v>
+      </c>
+      <c r="E110" t="s">
+        <v>1188</v>
+      </c>
+      <c r="F110" t="s">
+        <v>156</v>
+      </c>
+      <c r="G110" t="s">
+        <v>1189</v>
+      </c>
+      <c r="H110" t="s">
+        <v>49</v>
+      </c>
+      <c r="I110" t="s">
+        <v>1190</v>
+      </c>
+      <c r="J110" t="s">
+        <v>1191</v>
+      </c>
+      <c r="K110" t="s">
+        <v>422</v>
+      </c>
+      <c r="L110" t="s">
+        <v>876</v>
+      </c>
+      <c r="M110" t="s">
+        <v>53</v>
+      </c>
+      <c r="N110" t="s">
+        <v>54</v>
+      </c>
+      <c r="O110" t="s">
+        <v>139</v>
+      </c>
+      <c r="P110" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q110" t="s">
+        <v>76</v>
+      </c>
+      <c r="R110" t="s">
+        <v>578</v>
+      </c>
+      <c r="S110" t="s">
+        <v>49</v>
+      </c>
+      <c r="T110" t="s">
+        <v>579</v>
+      </c>
+      <c r="U110" t="s">
+        <v>57</v>
+      </c>
+      <c r="V110" t="s">
+        <v>57</v>
+      </c>
+      <c r="W110" t="s">
+        <v>163</v>
+      </c>
+      <c r="X110" t="s">
+        <v>580</v>
+      </c>
+      <c r="Y110" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z110" t="s">
+        <v>581</v>
+      </c>
+      <c r="AA110" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB110" t="s">
+        <v>1192</v>
+      </c>
+      <c r="AC110" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD110" t="s">
+        <v>230</v>
+      </c>
+      <c r="AE110" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF110" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG110" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH110" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI110" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ110" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK110" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL110" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM110" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN110" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO110" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP110" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="111" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>42</v>
+      </c>
+      <c r="B111" t="s">
+        <v>43</v>
+      </c>
+      <c r="C111" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D111" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E111" t="s">
+        <v>1196</v>
+      </c>
+      <c r="F111" t="s">
+        <v>235</v>
+      </c>
+      <c r="G111" t="s">
+        <v>1197</v>
+      </c>
+      <c r="H111" t="s">
+        <v>49</v>
+      </c>
+      <c r="I111" t="s">
+        <v>1198</v>
+      </c>
+      <c r="J111" t="s">
+        <v>1199</v>
+      </c>
+      <c r="K111" t="s">
+        <v>866</v>
+      </c>
+      <c r="L111" t="s">
+        <v>876</v>
+      </c>
+      <c r="M111" t="s">
+        <v>53</v>
+      </c>
+      <c r="N111" t="s">
+        <v>54</v>
+      </c>
+      <c r="O111" t="s">
+        <v>139</v>
+      </c>
+      <c r="P111" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q111" t="s">
+        <v>95</v>
+      </c>
+      <c r="R111" t="s">
+        <v>897</v>
+      </c>
+      <c r="S111" t="s">
+        <v>49</v>
+      </c>
+      <c r="T111" t="s">
+        <v>898</v>
+      </c>
+      <c r="U111" t="s">
+        <v>57</v>
+      </c>
+      <c r="V111" t="s">
+        <v>57</v>
+      </c>
+      <c r="W111" t="s">
+        <v>163</v>
+      </c>
+      <c r="X111" t="s">
+        <v>1048</v>
+      </c>
+      <c r="Y111" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z111" t="s">
+        <v>1049</v>
+      </c>
+      <c r="AA111" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB111" t="s">
+        <v>1200</v>
+      </c>
+      <c r="AC111" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD111" t="s">
+        <v>63</v>
+      </c>
+      <c r="AE111" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF111" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG111" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH111" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI111" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ111" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK111" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL111" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM111" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN111" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO111" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP111" t="s">
+        <v>1201</v>
+      </c>
+    </row>
+    <row r="112" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>42</v>
+      </c>
+      <c r="B112" t="s">
+        <v>43</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1202</v>
+      </c>
+      <c r="D112" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E112" t="s">
+        <v>1204</v>
+      </c>
+      <c r="F112" t="s">
+        <v>235</v>
+      </c>
+      <c r="G112" t="s">
+        <v>1197</v>
+      </c>
+      <c r="H112" t="s">
+        <v>1205</v>
+      </c>
+      <c r="I112" t="s">
+        <v>1205</v>
+      </c>
+      <c r="J112" t="s">
+        <v>1199</v>
+      </c>
+      <c r="K112" t="s">
+        <v>866</v>
+      </c>
+      <c r="L112" t="s">
+        <v>876</v>
+      </c>
+      <c r="M112" t="s">
+        <v>53</v>
+      </c>
+      <c r="N112" t="s">
+        <v>54</v>
+      </c>
+      <c r="O112" t="s">
+        <v>139</v>
+      </c>
+      <c r="P112" t="s">
+        <v>439</v>
+      </c>
+      <c r="Q112" t="s">
+        <v>95</v>
+      </c>
+      <c r="R112" t="s">
+        <v>283</v>
+      </c>
+      <c r="S112" t="s">
+        <v>49</v>
+      </c>
+      <c r="T112" t="s">
+        <v>284</v>
+      </c>
+      <c r="U112" t="s">
+        <v>57</v>
+      </c>
+      <c r="V112" t="s">
+        <v>57</v>
+      </c>
+      <c r="W112" t="s">
+        <v>163</v>
+      </c>
+      <c r="X112" t="s">
+        <v>923</v>
+      </c>
+      <c r="Y112" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z112" t="s">
+        <v>897</v>
+      </c>
+      <c r="AA112" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB112" t="s">
+        <v>1206</v>
+      </c>
+      <c r="AC112" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD112" t="s">
+        <v>498</v>
+      </c>
+      <c r="AE112" t="s">
+        <v>328</v>
+      </c>
+      <c r="AF112" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG112" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH112" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI112" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ112" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK112" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL112" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM112" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN112" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO112" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP112" t="s">
+        <v>1207</v>
+      </c>
+    </row>
+    <row r="113" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>42</v>
+      </c>
+      <c r="B113" t="s">
+        <v>43</v>
+      </c>
+      <c r="C113" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D113" t="s">
+        <v>1209</v>
+      </c>
+      <c r="E113" t="s">
+        <v>1210</v>
+      </c>
+      <c r="F113" t="s">
+        <v>89</v>
+      </c>
+      <c r="G113" t="s">
+        <v>347</v>
+      </c>
+      <c r="H113" t="s">
+        <v>1211</v>
+      </c>
+      <c r="I113" t="s">
+        <v>1211</v>
+      </c>
+      <c r="J113" t="s">
+        <v>349</v>
+      </c>
+      <c r="K113" t="s">
+        <v>876</v>
+      </c>
+      <c r="L113" t="s">
+        <v>876</v>
+      </c>
+      <c r="M113" t="s">
+        <v>53</v>
+      </c>
+      <c r="N113" t="s">
+        <v>54</v>
+      </c>
+      <c r="O113" t="s">
+        <v>55</v>
+      </c>
+      <c r="P113" t="s">
+        <v>319</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>76</v>
+      </c>
+      <c r="R113" t="s">
+        <v>482</v>
+      </c>
+      <c r="S113" t="s">
+        <v>49</v>
+      </c>
+      <c r="T113" t="s">
+        <v>511</v>
+      </c>
+      <c r="U113" t="s">
+        <v>57</v>
+      </c>
+      <c r="V113" t="s">
+        <v>57</v>
+      </c>
+      <c r="W113" t="s">
+        <v>257</v>
+      </c>
+      <c r="X113" t="s">
+        <v>481</v>
+      </c>
+      <c r="Y113" t="s">
+        <v>876</v>
+      </c>
+      <c r="Z113" t="s">
+        <v>512</v>
+      </c>
+      <c r="AA113" t="s">
+        <v>822</v>
+      </c>
+      <c r="AB113" t="s">
+        <v>719</v>
+      </c>
+      <c r="AC113" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD113" t="s">
+        <v>515</v>
+      </c>
+      <c r="AE113" t="s">
+        <v>311</v>
+      </c>
+      <c r="AF113" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG113" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH113" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI113" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ113" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK113" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL113" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM113" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN113" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO113" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP113" t="s">
+        <v>1212</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP101" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
📊 Actualizar CONSULTA_VENTA_PF.xlsx — 01-04-2026, 4:06:31 p. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_PF.xlsx
+++ b/datos/CONSULTA_VENTA_PF.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1210F783-412B-4AE0-A961-DAE578DA2515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{1210F783-412B-4AE0-A961-DAE578DA2515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F600A4C-811C-4744-8DB3-39192154BA39}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ParamQuery Pro" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ParamQuery Pro'!$A$1:$AP$113</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -2584,9 +2587,6 @@
     <t>29/03/2026</t>
   </si>
   <si>
-    <t>ERNESTO OLIVA</t>
-  </si>
-  <si>
     <t>1890756</t>
   </si>
   <si>
@@ -3659,6 +3659,9 @@
   </si>
   <si>
     <t>4175</t>
+  </si>
+  <si>
+    <t>Rodolfo Santana</t>
   </si>
 </sst>
 </file>
@@ -5466,7 +5469,7 @@
         <v>54</v>
       </c>
       <c r="O8" t="s">
-        <v>139</v>
+        <v>1212</v>
       </c>
       <c r="P8" t="s">
         <v>140</v>
@@ -5594,7 +5597,7 @@
         <v>54</v>
       </c>
       <c r="O9" t="s">
-        <v>139</v>
+        <v>1212</v>
       </c>
       <c r="P9" t="s">
         <v>140</v>
@@ -13658,7 +13661,7 @@
         <v>54</v>
       </c>
       <c r="O72" t="s">
-        <v>854</v>
+        <v>55</v>
       </c>
       <c r="P72" t="s">
         <v>55</v>
@@ -13673,7 +13676,7 @@
         <v>49</v>
       </c>
       <c r="T72" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="U72" t="s">
         <v>57</v>
@@ -13691,13 +13694,13 @@
         <v>853</v>
       </c>
       <c r="Z72" t="s">
+        <v>855</v>
+      </c>
+      <c r="AA72" t="s">
         <v>856</v>
       </c>
-      <c r="AA72" t="s">
+      <c r="AB72" t="s">
         <v>857</v>
-      </c>
-      <c r="AB72" t="s">
-        <v>858</v>
       </c>
       <c r="AC72" t="s">
         <v>774</v>
@@ -13739,7 +13742,7 @@
         <v>49</v>
       </c>
       <c r="AP72" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="73" spans="1:42" x14ac:dyDescent="0.3">
@@ -13750,34 +13753,34 @@
         <v>43</v>
       </c>
       <c r="C73" t="s">
+        <v>859</v>
+      </c>
+      <c r="D73" t="s">
         <v>860</v>
       </c>
-      <c r="D73" t="s">
+      <c r="E73" t="s">
         <v>861</v>
-      </c>
-      <c r="E73" t="s">
-        <v>862</v>
       </c>
       <c r="F73" t="s">
         <v>827</v>
       </c>
       <c r="G73" t="s">
+        <v>862</v>
+      </c>
+      <c r="H73" t="s">
+        <v>49</v>
+      </c>
+      <c r="I73" t="s">
         <v>863</v>
       </c>
-      <c r="H73" t="s">
-        <v>49</v>
-      </c>
-      <c r="I73" t="s">
+      <c r="J73" t="s">
         <v>864</v>
       </c>
-      <c r="J73" t="s">
+      <c r="K73" t="s">
         <v>865</v>
       </c>
-      <c r="K73" t="s">
-        <v>866</v>
-      </c>
       <c r="L73" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M73" t="s">
         <v>53</v>
@@ -13816,7 +13819,7 @@
         <v>481</v>
       </c>
       <c r="Y73" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Z73" t="s">
         <v>512</v>
@@ -13825,7 +13828,7 @@
         <v>569</v>
       </c>
       <c r="AB73" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="AC73" t="s">
         <v>774</v>
@@ -13867,7 +13870,7 @@
         <v>49</v>
       </c>
       <c r="AP73" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="74" spans="1:42" x14ac:dyDescent="0.3">
@@ -13878,34 +13881,34 @@
         <v>43</v>
       </c>
       <c r="C74" t="s">
+        <v>868</v>
+      </c>
+      <c r="D74" t="s">
         <v>869</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>870</v>
-      </c>
-      <c r="E74" t="s">
-        <v>871</v>
       </c>
       <c r="F74" t="s">
         <v>156</v>
       </c>
       <c r="G74" t="s">
+        <v>871</v>
+      </c>
+      <c r="H74" t="s">
         <v>872</v>
       </c>
-      <c r="H74" t="s">
+      <c r="I74" t="s">
         <v>873</v>
       </c>
-      <c r="I74" t="s">
+      <c r="J74" t="s">
         <v>874</v>
-      </c>
-      <c r="J74" t="s">
-        <v>875</v>
       </c>
       <c r="K74" t="s">
         <v>716</v>
       </c>
       <c r="L74" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M74" t="s">
         <v>53</v>
@@ -13944,7 +13947,7 @@
         <v>580</v>
       </c>
       <c r="Y74" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z74" t="s">
         <v>581</v>
@@ -13953,7 +13956,7 @@
         <v>148</v>
       </c>
       <c r="AB74" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="AC74" t="s">
         <v>774</v>
@@ -13995,7 +13998,7 @@
         <v>49</v>
       </c>
       <c r="AP74" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="75" spans="1:42" x14ac:dyDescent="0.3">
@@ -14006,34 +14009,34 @@
         <v>43</v>
       </c>
       <c r="C75" t="s">
+        <v>878</v>
+      </c>
+      <c r="D75" t="s">
         <v>879</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>880</v>
-      </c>
-      <c r="E75" t="s">
-        <v>881</v>
       </c>
       <c r="F75" t="s">
         <v>156</v>
       </c>
       <c r="G75" t="s">
+        <v>881</v>
+      </c>
+      <c r="H75" t="s">
+        <v>49</v>
+      </c>
+      <c r="I75" t="s">
         <v>882</v>
       </c>
-      <c r="H75" t="s">
-        <v>49</v>
-      </c>
-      <c r="I75" t="s">
+      <c r="J75" t="s">
         <v>883</v>
-      </c>
-      <c r="J75" t="s">
-        <v>884</v>
       </c>
       <c r="K75" t="s">
         <v>624</v>
       </c>
       <c r="L75" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M75" t="s">
         <v>53</v>
@@ -14057,7 +14060,7 @@
         <v>49</v>
       </c>
       <c r="T75" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="U75" t="s">
         <v>57</v>
@@ -14069,19 +14072,19 @@
         <v>163</v>
       </c>
       <c r="X75" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="Y75" t="s">
         <v>624</v>
       </c>
       <c r="Z75" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="AA75" t="s">
         <v>148</v>
       </c>
       <c r="AB75" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="AC75" t="s">
         <v>774</v>
@@ -14123,7 +14126,7 @@
         <v>49</v>
       </c>
       <c r="AP75" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="76" spans="1:42" x14ac:dyDescent="0.3">
@@ -14134,34 +14137,34 @@
         <v>43</v>
       </c>
       <c r="C76" t="s">
+        <v>888</v>
+      </c>
+      <c r="D76" t="s">
         <v>889</v>
       </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>890</v>
-      </c>
-      <c r="E76" t="s">
-        <v>891</v>
       </c>
       <c r="F76" t="s">
         <v>156</v>
       </c>
       <c r="G76" t="s">
+        <v>891</v>
+      </c>
+      <c r="H76" t="s">
         <v>892</v>
       </c>
-      <c r="H76" t="s">
+      <c r="I76" t="s">
+        <v>892</v>
+      </c>
+      <c r="J76" t="s">
         <v>893</v>
-      </c>
-      <c r="I76" t="s">
-        <v>893</v>
-      </c>
-      <c r="J76" t="s">
-        <v>894</v>
       </c>
       <c r="K76" t="s">
         <v>716</v>
       </c>
       <c r="L76" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M76" t="s">
         <v>53</v>
@@ -14209,7 +14212,7 @@
         <v>148</v>
       </c>
       <c r="AB76" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="AC76" t="s">
         <v>774</v>
@@ -14251,7 +14254,7 @@
         <v>49</v>
       </c>
       <c r="AP76" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="77" spans="1:42" x14ac:dyDescent="0.3">
@@ -14289,7 +14292,7 @@
         <v>844</v>
       </c>
       <c r="L77" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M77" t="s">
         <v>53</v>
@@ -14307,37 +14310,37 @@
         <v>76</v>
       </c>
       <c r="R77" t="s">
+        <v>896</v>
+      </c>
+      <c r="S77" t="s">
+        <v>49</v>
+      </c>
+      <c r="T77" t="s">
         <v>897</v>
       </c>
-      <c r="S77" t="s">
-        <v>49</v>
-      </c>
-      <c r="T77" t="s">
+      <c r="U77" t="s">
+        <v>57</v>
+      </c>
+      <c r="V77" t="s">
+        <v>57</v>
+      </c>
+      <c r="W77" t="s">
         <v>898</v>
       </c>
-      <c r="U77" t="s">
-        <v>57</v>
-      </c>
-      <c r="V77" t="s">
-        <v>57</v>
-      </c>
-      <c r="W77" t="s">
+      <c r="X77" t="s">
         <v>899</v>
       </c>
-      <c r="X77" t="s">
+      <c r="Y77" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z77" t="s">
         <v>900</v>
-      </c>
-      <c r="Y77" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z77" t="s">
-        <v>901</v>
       </c>
       <c r="AA77" t="s">
         <v>354</v>
       </c>
       <c r="AB77" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="AC77" t="s">
         <v>774</v>
@@ -14379,7 +14382,7 @@
         <v>49</v>
       </c>
       <c r="AP77" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="78" spans="1:42" x14ac:dyDescent="0.3">
@@ -14417,7 +14420,7 @@
         <v>844</v>
       </c>
       <c r="L78" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M78" t="s">
         <v>53</v>
@@ -14435,37 +14438,37 @@
         <v>76</v>
       </c>
       <c r="R78" t="s">
+        <v>896</v>
+      </c>
+      <c r="S78" t="s">
+        <v>49</v>
+      </c>
+      <c r="T78" t="s">
         <v>897</v>
       </c>
-      <c r="S78" t="s">
-        <v>49</v>
-      </c>
-      <c r="T78" t="s">
+      <c r="U78" t="s">
+        <v>57</v>
+      </c>
+      <c r="V78" t="s">
+        <v>57</v>
+      </c>
+      <c r="W78" t="s">
         <v>898</v>
       </c>
-      <c r="U78" t="s">
-        <v>57</v>
-      </c>
-      <c r="V78" t="s">
-        <v>57</v>
-      </c>
-      <c r="W78" t="s">
+      <c r="X78" t="s">
         <v>899</v>
       </c>
-      <c r="X78" t="s">
+      <c r="Y78" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z78" t="s">
         <v>900</v>
-      </c>
-      <c r="Y78" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z78" t="s">
-        <v>901</v>
       </c>
       <c r="AA78" t="s">
         <v>226</v>
       </c>
       <c r="AB78" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="AC78" t="s">
         <v>774</v>
@@ -14507,7 +14510,7 @@
         <v>49</v>
       </c>
       <c r="AP78" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="79" spans="1:42" x14ac:dyDescent="0.3">
@@ -14518,34 +14521,34 @@
         <v>43</v>
       </c>
       <c r="C79" t="s">
+        <v>904</v>
+      </c>
+      <c r="D79" t="s">
         <v>905</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
         <v>906</v>
-      </c>
-      <c r="E79" t="s">
-        <v>907</v>
       </c>
       <c r="F79" t="s">
         <v>89</v>
       </c>
       <c r="G79" t="s">
+        <v>907</v>
+      </c>
+      <c r="H79" t="s">
         <v>908</v>
       </c>
-      <c r="H79" t="s">
+      <c r="I79" t="s">
+        <v>908</v>
+      </c>
+      <c r="J79" t="s">
         <v>909</v>
       </c>
-      <c r="I79" t="s">
-        <v>909</v>
-      </c>
-      <c r="J79" t="s">
-        <v>910</v>
-      </c>
       <c r="K79" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L79" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M79" t="s">
         <v>53</v>
@@ -14563,13 +14566,13 @@
         <v>626</v>
       </c>
       <c r="R79" t="s">
+        <v>910</v>
+      </c>
+      <c r="S79" t="s">
+        <v>49</v>
+      </c>
+      <c r="T79" t="s">
         <v>911</v>
-      </c>
-      <c r="S79" t="s">
-        <v>49</v>
-      </c>
-      <c r="T79" t="s">
-        <v>912</v>
       </c>
       <c r="U79" t="s">
         <v>57</v>
@@ -14581,19 +14584,19 @@
         <v>163</v>
       </c>
       <c r="X79" t="s">
+        <v>912</v>
+      </c>
+      <c r="Y79" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z79" t="s">
         <v>913</v>
-      </c>
-      <c r="Y79" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z79" t="s">
-        <v>914</v>
       </c>
       <c r="AA79" t="s">
         <v>148</v>
       </c>
       <c r="AB79" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="AC79" t="s">
         <v>774</v>
@@ -14635,7 +14638,7 @@
         <v>49</v>
       </c>
       <c r="AP79" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="80" spans="1:42" x14ac:dyDescent="0.3">
@@ -14646,28 +14649,28 @@
         <v>43</v>
       </c>
       <c r="C80" t="s">
+        <v>916</v>
+      </c>
+      <c r="D80" t="s">
         <v>917</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>918</v>
-      </c>
-      <c r="E80" t="s">
-        <v>919</v>
       </c>
       <c r="F80" t="s">
         <v>89</v>
       </c>
       <c r="G80" t="s">
+        <v>919</v>
+      </c>
+      <c r="H80" t="s">
+        <v>49</v>
+      </c>
+      <c r="I80" t="s">
         <v>920</v>
       </c>
-      <c r="H80" t="s">
-        <v>49</v>
-      </c>
-      <c r="I80" t="s">
+      <c r="J80" t="s">
         <v>921</v>
-      </c>
-      <c r="J80" t="s">
-        <v>922</v>
       </c>
       <c r="K80" t="s">
         <v>831</v>
@@ -14691,13 +14694,13 @@
         <v>240</v>
       </c>
       <c r="R80" t="s">
+        <v>896</v>
+      </c>
+      <c r="S80" t="s">
+        <v>49</v>
+      </c>
+      <c r="T80" t="s">
         <v>897</v>
-      </c>
-      <c r="S80" t="s">
-        <v>49</v>
-      </c>
-      <c r="T80" t="s">
-        <v>898</v>
       </c>
       <c r="U80" t="s">
         <v>57</v>
@@ -14709,19 +14712,19 @@
         <v>257</v>
       </c>
       <c r="X80" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="Y80" t="s">
         <v>817</v>
       </c>
       <c r="Z80" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="AA80" t="s">
         <v>440</v>
       </c>
       <c r="AB80" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="AC80" t="s">
         <v>774</v>
@@ -14763,7 +14766,7 @@
         <v>49</v>
       </c>
       <c r="AP80" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="81" spans="1:42" x14ac:dyDescent="0.3">
@@ -14774,28 +14777,28 @@
         <v>43</v>
       </c>
       <c r="C81" t="s">
+        <v>926</v>
+      </c>
+      <c r="D81" t="s">
         <v>927</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>928</v>
-      </c>
-      <c r="E81" t="s">
-        <v>929</v>
       </c>
       <c r="F81" t="s">
         <v>156</v>
       </c>
       <c r="G81" t="s">
+        <v>929</v>
+      </c>
+      <c r="H81" t="s">
+        <v>49</v>
+      </c>
+      <c r="I81" t="s">
         <v>930</v>
       </c>
-      <c r="H81" t="s">
-        <v>49</v>
-      </c>
-      <c r="I81" t="s">
+      <c r="J81" t="s">
         <v>931</v>
-      </c>
-      <c r="J81" t="s">
-        <v>932</v>
       </c>
       <c r="K81" t="s">
         <v>831</v>
@@ -14891,7 +14894,7 @@
         <v>49</v>
       </c>
       <c r="AP81" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="82" spans="1:42" x14ac:dyDescent="0.3">
@@ -14902,28 +14905,28 @@
         <v>43</v>
       </c>
       <c r="C82" t="s">
+        <v>933</v>
+      </c>
+      <c r="D82" t="s">
         <v>934</v>
       </c>
-      <c r="D82" t="s">
+      <c r="E82" t="s">
         <v>935</v>
-      </c>
-      <c r="E82" t="s">
-        <v>936</v>
       </c>
       <c r="F82" t="s">
         <v>156</v>
       </c>
       <c r="G82" t="s">
+        <v>936</v>
+      </c>
+      <c r="H82" t="s">
+        <v>49</v>
+      </c>
+      <c r="I82" t="s">
         <v>937</v>
       </c>
-      <c r="H82" t="s">
-        <v>49</v>
-      </c>
-      <c r="I82" t="s">
+      <c r="J82" t="s">
         <v>938</v>
-      </c>
-      <c r="J82" t="s">
-        <v>939</v>
       </c>
       <c r="K82" t="s">
         <v>304</v>
@@ -15019,7 +15022,7 @@
         <v>49</v>
       </c>
       <c r="AP82" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="83" spans="1:42" x14ac:dyDescent="0.3">
@@ -15030,34 +15033,34 @@
         <v>43</v>
       </c>
       <c r="C83" t="s">
+        <v>940</v>
+      </c>
+      <c r="D83" t="s">
         <v>941</v>
       </c>
-      <c r="D83" t="s">
+      <c r="E83" t="s">
         <v>942</v>
-      </c>
-      <c r="E83" t="s">
-        <v>943</v>
       </c>
       <c r="F83" t="s">
         <v>333</v>
       </c>
       <c r="G83" t="s">
+        <v>943</v>
+      </c>
+      <c r="H83" t="s">
         <v>944</v>
       </c>
-      <c r="H83" t="s">
+      <c r="I83" t="s">
+        <v>944</v>
+      </c>
+      <c r="J83" t="s">
         <v>945</v>
-      </c>
-      <c r="I83" t="s">
-        <v>945</v>
-      </c>
-      <c r="J83" t="s">
-        <v>946</v>
       </c>
       <c r="K83" t="s">
         <v>177</v>
       </c>
       <c r="L83" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M83" t="s">
         <v>53</v>
@@ -15075,13 +15078,13 @@
         <v>211</v>
       </c>
       <c r="R83" t="s">
+        <v>946</v>
+      </c>
+      <c r="S83" t="s">
+        <v>49</v>
+      </c>
+      <c r="T83" t="s">
         <v>947</v>
-      </c>
-      <c r="S83" t="s">
-        <v>49</v>
-      </c>
-      <c r="T83" t="s">
-        <v>948</v>
       </c>
       <c r="U83" t="s">
         <v>57</v>
@@ -15093,25 +15096,25 @@
         <v>163</v>
       </c>
       <c r="X83" t="s">
+        <v>948</v>
+      </c>
+      <c r="Y83" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z83" t="s">
         <v>949</v>
-      </c>
-      <c r="Y83" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z83" t="s">
-        <v>950</v>
       </c>
       <c r="AA83" t="s">
         <v>148</v>
       </c>
       <c r="AB83" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="AC83" t="s">
         <v>774</v>
       </c>
       <c r="AD83" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="AE83" t="s">
         <v>126</v>
@@ -15147,7 +15150,7 @@
         <v>49</v>
       </c>
       <c r="AP83" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="84" spans="1:42" x14ac:dyDescent="0.3">
@@ -15158,34 +15161,34 @@
         <v>43</v>
       </c>
       <c r="C84" t="s">
+        <v>953</v>
+      </c>
+      <c r="D84" t="s">
         <v>954</v>
       </c>
-      <c r="D84" t="s">
+      <c r="E84" t="s">
         <v>955</v>
       </c>
-      <c r="E84" t="s">
+      <c r="F84" t="s">
         <v>956</v>
       </c>
-      <c r="F84" t="s">
+      <c r="G84" t="s">
         <v>957</v>
       </c>
-      <c r="G84" t="s">
+      <c r="H84" t="s">
         <v>958</v>
       </c>
-      <c r="H84" t="s">
+      <c r="I84" t="s">
+        <v>958</v>
+      </c>
+      <c r="J84" t="s">
         <v>959</v>
       </c>
-      <c r="I84" t="s">
-        <v>959</v>
-      </c>
-      <c r="J84" t="s">
-        <v>960</v>
-      </c>
       <c r="K84" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L84" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M84" t="s">
         <v>53</v>
@@ -15194,22 +15197,22 @@
         <v>54</v>
       </c>
       <c r="O84" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="P84" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="Q84" t="s">
         <v>76</v>
       </c>
       <c r="R84" t="s">
+        <v>961</v>
+      </c>
+      <c r="S84" t="s">
+        <v>49</v>
+      </c>
+      <c r="T84" t="s">
         <v>962</v>
-      </c>
-      <c r="S84" t="s">
-        <v>49</v>
-      </c>
-      <c r="T84" t="s">
-        <v>963</v>
       </c>
       <c r="U84" t="s">
         <v>57</v>
@@ -15221,25 +15224,25 @@
         <v>163</v>
       </c>
       <c r="X84" t="s">
+        <v>963</v>
+      </c>
+      <c r="Y84" t="s">
+        <v>865</v>
+      </c>
+      <c r="Z84" t="s">
         <v>964</v>
-      </c>
-      <c r="Y84" t="s">
-        <v>866</v>
-      </c>
-      <c r="Z84" t="s">
-        <v>965</v>
       </c>
       <c r="AA84" t="s">
         <v>260</v>
       </c>
       <c r="AB84" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="AC84" t="s">
         <v>774</v>
       </c>
       <c r="AD84" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="AE84" t="s">
         <v>456</v>
@@ -15275,7 +15278,7 @@
         <v>49</v>
       </c>
       <c r="AP84" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="85" spans="1:42" x14ac:dyDescent="0.3">
@@ -15286,34 +15289,34 @@
         <v>43</v>
       </c>
       <c r="C85" t="s">
+        <v>968</v>
+      </c>
+      <c r="D85" t="s">
         <v>969</v>
       </c>
-      <c r="D85" t="s">
+      <c r="E85" t="s">
         <v>970</v>
       </c>
-      <c r="E85" t="s">
+      <c r="F85" t="s">
         <v>971</v>
       </c>
-      <c r="F85" t="s">
+      <c r="G85" t="s">
         <v>972</v>
       </c>
-      <c r="G85" t="s">
+      <c r="H85" t="s">
         <v>973</v>
       </c>
-      <c r="H85" t="s">
+      <c r="I85" t="s">
+        <v>973</v>
+      </c>
+      <c r="J85" t="s">
         <v>974</v>
       </c>
-      <c r="I85" t="s">
-        <v>974</v>
-      </c>
-      <c r="J85" t="s">
-        <v>975</v>
-      </c>
       <c r="K85" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L85" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M85" t="s">
         <v>53</v>
@@ -15346,22 +15349,22 @@
         <v>57</v>
       </c>
       <c r="W85" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="X85" t="s">
         <v>200</v>
       </c>
       <c r="Y85" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z85" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="AA85" t="s">
         <v>178</v>
       </c>
       <c r="AB85" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AC85" t="s">
         <v>774</v>
@@ -15403,7 +15406,7 @@
         <v>49</v>
       </c>
       <c r="AP85" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="86" spans="1:42" x14ac:dyDescent="0.3">
@@ -15414,34 +15417,34 @@
         <v>43</v>
       </c>
       <c r="C86" t="s">
+        <v>978</v>
+      </c>
+      <c r="D86" t="s">
         <v>979</v>
       </c>
-      <c r="D86" t="s">
+      <c r="E86" t="s">
         <v>980</v>
       </c>
-      <c r="E86" t="s">
-        <v>981</v>
-      </c>
       <c r="F86" t="s">
+        <v>971</v>
+      </c>
+      <c r="G86" t="s">
         <v>972</v>
       </c>
-      <c r="G86" t="s">
+      <c r="H86" t="s">
         <v>973</v>
       </c>
-      <c r="H86" t="s">
+      <c r="I86" t="s">
+        <v>973</v>
+      </c>
+      <c r="J86" t="s">
         <v>974</v>
       </c>
-      <c r="I86" t="s">
-        <v>974</v>
-      </c>
-      <c r="J86" t="s">
-        <v>975</v>
-      </c>
       <c r="K86" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L86" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M86" t="s">
         <v>53</v>
@@ -15474,22 +15477,22 @@
         <v>57</v>
       </c>
       <c r="W86" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="X86" t="s">
         <v>200</v>
       </c>
       <c r="Y86" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z86" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="AA86" t="s">
         <v>178</v>
       </c>
       <c r="AB86" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AC86" t="s">
         <v>774</v>
@@ -15531,7 +15534,7 @@
         <v>49</v>
       </c>
       <c r="AP86" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="87" spans="1:42" x14ac:dyDescent="0.3">
@@ -15542,34 +15545,34 @@
         <v>43</v>
       </c>
       <c r="C87" t="s">
+        <v>982</v>
+      </c>
+      <c r="D87" t="s">
         <v>983</v>
       </c>
-      <c r="D87" t="s">
+      <c r="E87" t="s">
         <v>984</v>
-      </c>
-      <c r="E87" t="s">
-        <v>985</v>
       </c>
       <c r="F87" t="s">
         <v>736</v>
       </c>
       <c r="G87" t="s">
+        <v>985</v>
+      </c>
+      <c r="H87" t="s">
+        <v>49</v>
+      </c>
+      <c r="I87" t="s">
         <v>986</v>
       </c>
-      <c r="H87" t="s">
-        <v>49</v>
-      </c>
-      <c r="I87" t="s">
+      <c r="J87" t="s">
         <v>987</v>
-      </c>
-      <c r="J87" t="s">
-        <v>988</v>
       </c>
       <c r="K87" t="s">
         <v>684</v>
       </c>
       <c r="L87" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M87" t="s">
         <v>53</v>
@@ -15608,7 +15611,7 @@
         <v>580</v>
       </c>
       <c r="Y87" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z87" t="s">
         <v>581</v>
@@ -15617,7 +15620,7 @@
         <v>260</v>
       </c>
       <c r="AB87" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="AC87" t="s">
         <v>774</v>
@@ -15659,7 +15662,7 @@
         <v>49</v>
       </c>
       <c r="AP87" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
     </row>
     <row r="88" spans="1:42" x14ac:dyDescent="0.3">
@@ -15670,34 +15673,34 @@
         <v>43</v>
       </c>
       <c r="C88" t="s">
+        <v>990</v>
+      </c>
+      <c r="D88" t="s">
         <v>991</v>
       </c>
-      <c r="D88" t="s">
+      <c r="E88" t="s">
         <v>992</v>
-      </c>
-      <c r="E88" t="s">
-        <v>993</v>
       </c>
       <c r="F88" t="s">
         <v>840</v>
       </c>
       <c r="G88" t="s">
+        <v>993</v>
+      </c>
+      <c r="H88" t="s">
+        <v>49</v>
+      </c>
+      <c r="I88" t="s">
         <v>994</v>
       </c>
-      <c r="H88" t="s">
-        <v>49</v>
-      </c>
-      <c r="I88" t="s">
+      <c r="J88" t="s">
         <v>995</v>
-      </c>
-      <c r="J88" t="s">
-        <v>996</v>
       </c>
       <c r="K88" t="s">
         <v>794</v>
       </c>
       <c r="L88" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M88" t="s">
         <v>53</v>
@@ -15709,7 +15712,7 @@
         <v>398</v>
       </c>
       <c r="P88" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="Q88" t="s">
         <v>240</v>
@@ -15736,7 +15739,7 @@
         <v>538</v>
       </c>
       <c r="Y88" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z88" t="s">
         <v>350</v>
@@ -15745,7 +15748,7 @@
         <v>342</v>
       </c>
       <c r="AB88" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="AC88" t="s">
         <v>774</v>
@@ -15787,7 +15790,7 @@
         <v>49</v>
       </c>
       <c r="AP88" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="89" spans="1:42" x14ac:dyDescent="0.3">
@@ -15798,34 +15801,34 @@
         <v>43</v>
       </c>
       <c r="C89" t="s">
+        <v>999</v>
+      </c>
+      <c r="D89" t="s">
         <v>1000</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
         <v>1001</v>
       </c>
-      <c r="E89" t="s">
+      <c r="F89" t="s">
         <v>1002</v>
       </c>
-      <c r="F89" t="s">
+      <c r="G89" t="s">
         <v>1003</v>
       </c>
-      <c r="G89" t="s">
+      <c r="H89" t="s">
+        <v>49</v>
+      </c>
+      <c r="I89" t="s">
         <v>1004</v>
       </c>
-      <c r="H89" t="s">
-        <v>49</v>
-      </c>
-      <c r="I89" t="s">
+      <c r="J89" t="s">
         <v>1005</v>
-      </c>
-      <c r="J89" t="s">
-        <v>1006</v>
       </c>
       <c r="K89" t="s">
         <v>844</v>
       </c>
       <c r="L89" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M89" t="s">
         <v>53</v>
@@ -15843,13 +15846,13 @@
         <v>142</v>
       </c>
       <c r="R89" t="s">
+        <v>1006</v>
+      </c>
+      <c r="S89" t="s">
+        <v>49</v>
+      </c>
+      <c r="T89" t="s">
         <v>1007</v>
-      </c>
-      <c r="S89" t="s">
-        <v>49</v>
-      </c>
-      <c r="T89" t="s">
-        <v>1008</v>
       </c>
       <c r="U89" t="s">
         <v>57</v>
@@ -15861,19 +15864,19 @@
         <v>163</v>
       </c>
       <c r="X89" t="s">
+        <v>1008</v>
+      </c>
+      <c r="Y89" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z89" t="s">
         <v>1009</v>
-      </c>
-      <c r="Y89" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z89" t="s">
-        <v>1010</v>
       </c>
       <c r="AA89" t="s">
         <v>178</v>
       </c>
       <c r="AB89" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="AC89" t="s">
         <v>774</v>
@@ -15915,7 +15918,7 @@
         <v>49</v>
       </c>
       <c r="AP89" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="90" spans="1:42" x14ac:dyDescent="0.3">
@@ -15926,28 +15929,28 @@
         <v>43</v>
       </c>
       <c r="C90" t="s">
+        <v>1012</v>
+      </c>
+      <c r="D90" t="s">
         <v>1013</v>
       </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
         <v>1014</v>
-      </c>
-      <c r="E90" t="s">
-        <v>1015</v>
       </c>
       <c r="F90" t="s">
         <v>827</v>
       </c>
       <c r="G90" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H90" t="s">
         <v>1016</v>
       </c>
-      <c r="H90" t="s">
+      <c r="I90" t="s">
+        <v>1016</v>
+      </c>
+      <c r="J90" t="s">
         <v>1017</v>
-      </c>
-      <c r="I90" t="s">
-        <v>1017</v>
-      </c>
-      <c r="J90" t="s">
-        <v>1018</v>
       </c>
       <c r="K90" t="s">
         <v>659</v>
@@ -16001,7 +16004,7 @@
         <v>148</v>
       </c>
       <c r="AB90" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="AC90" t="s">
         <v>774</v>
@@ -16043,7 +16046,7 @@
         <v>49</v>
       </c>
       <c r="AP90" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="91" spans="1:42" x14ac:dyDescent="0.3">
@@ -16054,34 +16057,34 @@
         <v>43</v>
       </c>
       <c r="C91" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D91" t="s">
         <v>1021</v>
       </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
         <v>1022</v>
       </c>
-      <c r="E91" t="s">
-        <v>1023</v>
-      </c>
       <c r="F91" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G91" t="s">
         <v>1003</v>
       </c>
-      <c r="G91" t="s">
+      <c r="H91" t="s">
+        <v>863</v>
+      </c>
+      <c r="I91" t="s">
         <v>1004</v>
       </c>
-      <c r="H91" t="s">
-        <v>864</v>
-      </c>
-      <c r="I91" t="s">
+      <c r="J91" t="s">
         <v>1005</v>
-      </c>
-      <c r="J91" t="s">
-        <v>1006</v>
       </c>
       <c r="K91" t="s">
         <v>844</v>
       </c>
       <c r="L91" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M91" t="s">
         <v>53</v>
@@ -16099,13 +16102,13 @@
         <v>142</v>
       </c>
       <c r="R91" t="s">
+        <v>1006</v>
+      </c>
+      <c r="S91" t="s">
+        <v>49</v>
+      </c>
+      <c r="T91" t="s">
         <v>1007</v>
-      </c>
-      <c r="S91" t="s">
-        <v>49</v>
-      </c>
-      <c r="T91" t="s">
-        <v>1008</v>
       </c>
       <c r="U91" t="s">
         <v>57</v>
@@ -16117,19 +16120,19 @@
         <v>163</v>
       </c>
       <c r="X91" t="s">
+        <v>1008</v>
+      </c>
+      <c r="Y91" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z91" t="s">
         <v>1009</v>
-      </c>
-      <c r="Y91" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z91" t="s">
-        <v>1010</v>
       </c>
       <c r="AA91" t="s">
         <v>178</v>
       </c>
       <c r="AB91" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="AC91" t="s">
         <v>774</v>
@@ -16171,7 +16174,7 @@
         <v>49</v>
       </c>
       <c r="AP91" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="92" spans="1:42" x14ac:dyDescent="0.3">
@@ -16182,34 +16185,34 @@
         <v>43</v>
       </c>
       <c r="C92" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D92" t="s">
         <v>1025</v>
       </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
         <v>1026</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F92" t="s">
         <v>1027</v>
       </c>
-      <c r="F92" t="s">
+      <c r="G92" t="s">
         <v>1028</v>
       </c>
-      <c r="G92" t="s">
+      <c r="H92" t="s">
+        <v>49</v>
+      </c>
+      <c r="I92" t="s">
         <v>1029</v>
       </c>
-      <c r="H92" t="s">
-        <v>49</v>
-      </c>
-      <c r="I92" t="s">
+      <c r="J92" t="s">
         <v>1030</v>
       </c>
-      <c r="J92" t="s">
-        <v>1031</v>
-      </c>
       <c r="K92" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L92" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M92" t="s">
         <v>53</v>
@@ -16221,7 +16224,7 @@
         <v>590</v>
       </c>
       <c r="P92" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="Q92" t="s">
         <v>211</v>
@@ -16248,7 +16251,7 @@
         <v>538</v>
       </c>
       <c r="Y92" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z92" t="s">
         <v>350</v>
@@ -16299,7 +16302,7 @@
         <v>49</v>
       </c>
       <c r="AP92" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="93" spans="1:42" x14ac:dyDescent="0.3">
@@ -16310,34 +16313,34 @@
         <v>43</v>
       </c>
       <c r="C93" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D93" t="s">
         <v>1034</v>
       </c>
-      <c r="D93" t="s">
+      <c r="E93" t="s">
         <v>1035</v>
-      </c>
-      <c r="E93" t="s">
-        <v>1036</v>
       </c>
       <c r="F93" t="s">
         <v>371</v>
       </c>
       <c r="G93" t="s">
+        <v>1036</v>
+      </c>
+      <c r="H93" t="s">
+        <v>49</v>
+      </c>
+      <c r="I93" t="s">
         <v>1037</v>
       </c>
-      <c r="H93" t="s">
-        <v>49</v>
-      </c>
-      <c r="I93" t="s">
+      <c r="J93" t="s">
         <v>1038</v>
       </c>
-      <c r="J93" t="s">
-        <v>1039</v>
-      </c>
       <c r="K93" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L93" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M93" t="s">
         <v>53</v>
@@ -16349,7 +16352,7 @@
         <v>55</v>
       </c>
       <c r="P93" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="Q93" t="s">
         <v>211</v>
@@ -16376,7 +16379,7 @@
         <v>538</v>
       </c>
       <c r="Y93" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z93" t="s">
         <v>161</v>
@@ -16427,7 +16430,7 @@
         <v>49</v>
       </c>
       <c r="AP93" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="94" spans="1:42" x14ac:dyDescent="0.3">
@@ -16438,34 +16441,34 @@
         <v>43</v>
       </c>
       <c r="C94" t="s">
+        <v>1041</v>
+      </c>
+      <c r="D94" t="s">
         <v>1042</v>
       </c>
-      <c r="D94" t="s">
+      <c r="E94" t="s">
         <v>1043</v>
-      </c>
-      <c r="E94" t="s">
-        <v>1044</v>
       </c>
       <c r="F94" t="s">
         <v>333</v>
       </c>
       <c r="G94" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H94" t="s">
         <v>1045</v>
       </c>
-      <c r="H94" t="s">
+      <c r="I94" t="s">
+        <v>1045</v>
+      </c>
+      <c r="J94" t="s">
         <v>1046</v>
-      </c>
-      <c r="I94" t="s">
-        <v>1046</v>
-      </c>
-      <c r="J94" t="s">
-        <v>1047</v>
       </c>
       <c r="K94" t="s">
         <v>567</v>
       </c>
       <c r="L94" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M94" t="s">
         <v>53</v>
@@ -16483,13 +16486,13 @@
         <v>211</v>
       </c>
       <c r="R94" t="s">
+        <v>896</v>
+      </c>
+      <c r="S94" t="s">
+        <v>49</v>
+      </c>
+      <c r="T94" t="s">
         <v>897</v>
-      </c>
-      <c r="S94" t="s">
-        <v>49</v>
-      </c>
-      <c r="T94" t="s">
-        <v>898</v>
       </c>
       <c r="U94" t="s">
         <v>57</v>
@@ -16501,19 +16504,19 @@
         <v>163</v>
       </c>
       <c r="X94" t="s">
+        <v>1047</v>
+      </c>
+      <c r="Y94" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z94" t="s">
         <v>1048</v>
-      </c>
-      <c r="Y94" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z94" t="s">
-        <v>1049</v>
       </c>
       <c r="AA94" t="s">
         <v>184</v>
       </c>
       <c r="AB94" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="AC94" t="s">
         <v>774</v>
@@ -16555,7 +16558,7 @@
         <v>49</v>
       </c>
       <c r="AP94" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="95" spans="1:42" x14ac:dyDescent="0.3">
@@ -16566,34 +16569,34 @@
         <v>43</v>
       </c>
       <c r="C95" t="s">
+        <v>1051</v>
+      </c>
+      <c r="D95" t="s">
         <v>1052</v>
       </c>
-      <c r="D95" t="s">
+      <c r="E95" t="s">
         <v>1053</v>
-      </c>
-      <c r="E95" t="s">
-        <v>1054</v>
       </c>
       <c r="F95" t="s">
         <v>333</v>
       </c>
       <c r="G95" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="H95" t="s">
+        <v>1054</v>
+      </c>
+      <c r="I95" t="s">
+        <v>1054</v>
+      </c>
+      <c r="J95" t="s">
         <v>1055</v>
-      </c>
-      <c r="I95" t="s">
-        <v>1055</v>
-      </c>
-      <c r="J95" t="s">
-        <v>1056</v>
       </c>
       <c r="K95" t="s">
         <v>567</v>
       </c>
       <c r="L95" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M95" t="s">
         <v>53</v>
@@ -16632,7 +16635,7 @@
         <v>243</v>
       </c>
       <c r="Y95" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z95" t="s">
         <v>244</v>
@@ -16641,7 +16644,7 @@
         <v>822</v>
       </c>
       <c r="AB95" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="AC95" t="s">
         <v>774</v>
@@ -16683,7 +16686,7 @@
         <v>49</v>
       </c>
       <c r="AP95" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="96" spans="1:42" x14ac:dyDescent="0.3">
@@ -16694,34 +16697,34 @@
         <v>43</v>
       </c>
       <c r="C96" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D96" t="s">
         <v>1059</v>
       </c>
-      <c r="D96" t="s">
+      <c r="E96" t="s">
         <v>1060</v>
       </c>
-      <c r="E96" t="s">
+      <c r="F96" t="s">
         <v>1061</v>
       </c>
-      <c r="F96" t="s">
+      <c r="G96" t="s">
         <v>1062</v>
       </c>
-      <c r="G96" t="s">
+      <c r="H96" t="s">
         <v>1063</v>
       </c>
-      <c r="H96" t="s">
+      <c r="I96" t="s">
         <v>1064</v>
       </c>
-      <c r="I96" t="s">
+      <c r="J96" t="s">
         <v>1065</v>
-      </c>
-      <c r="J96" t="s">
-        <v>1066</v>
       </c>
       <c r="K96" t="s">
         <v>465</v>
       </c>
       <c r="L96" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M96" t="s">
         <v>53</v>
@@ -16757,19 +16760,19 @@
         <v>163</v>
       </c>
       <c r="X96" t="s">
+        <v>1066</v>
+      </c>
+      <c r="Y96" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z96" t="s">
         <v>1067</v>
-      </c>
-      <c r="Y96" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z96" t="s">
-        <v>1068</v>
       </c>
       <c r="AA96" t="s">
         <v>354</v>
       </c>
       <c r="AB96" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="AC96" t="s">
         <v>774</v>
@@ -16811,7 +16814,7 @@
         <v>49</v>
       </c>
       <c r="AP96" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="97" spans="1:42" x14ac:dyDescent="0.3">
@@ -16822,34 +16825,34 @@
         <v>43</v>
       </c>
       <c r="C97" t="s">
+        <v>1070</v>
+      </c>
+      <c r="D97" t="s">
         <v>1071</v>
       </c>
-      <c r="D97" t="s">
+      <c r="E97" t="s">
         <v>1072</v>
-      </c>
-      <c r="E97" t="s">
-        <v>1073</v>
       </c>
       <c r="F97" t="s">
         <v>235</v>
       </c>
       <c r="G97" t="s">
+        <v>1073</v>
+      </c>
+      <c r="H97" t="s">
+        <v>49</v>
+      </c>
+      <c r="I97" t="s">
         <v>1074</v>
       </c>
-      <c r="H97" t="s">
-        <v>49</v>
-      </c>
-      <c r="I97" t="s">
+      <c r="J97" t="s">
         <v>1075</v>
-      </c>
-      <c r="J97" t="s">
-        <v>1076</v>
       </c>
       <c r="K97" t="s">
         <v>844</v>
       </c>
       <c r="L97" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M97" t="s">
         <v>53</v>
@@ -16861,7 +16864,7 @@
         <v>398</v>
       </c>
       <c r="P97" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="Q97" t="s">
         <v>211</v>
@@ -16885,25 +16888,25 @@
         <v>163</v>
       </c>
       <c r="X97" t="s">
+        <v>1077</v>
+      </c>
+      <c r="Y97" t="s">
+        <v>865</v>
+      </c>
+      <c r="Z97" t="s">
         <v>1078</v>
-      </c>
-      <c r="Y97" t="s">
-        <v>866</v>
-      </c>
-      <c r="Z97" t="s">
-        <v>1079</v>
       </c>
       <c r="AA97" t="s">
         <v>95</v>
       </c>
       <c r="AB97" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="AC97" t="s">
         <v>774</v>
       </c>
       <c r="AD97" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="AE97" t="s">
         <v>126</v>
@@ -16939,7 +16942,7 @@
         <v>49</v>
       </c>
       <c r="AP97" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="98" spans="1:42" x14ac:dyDescent="0.3">
@@ -16950,34 +16953,34 @@
         <v>43</v>
       </c>
       <c r="C98" t="s">
+        <v>1081</v>
+      </c>
+      <c r="D98" t="s">
         <v>1082</v>
       </c>
-      <c r="D98" t="s">
+      <c r="E98" t="s">
         <v>1083</v>
-      </c>
-      <c r="E98" t="s">
-        <v>1084</v>
       </c>
       <c r="F98" t="s">
         <v>251</v>
       </c>
       <c r="G98" t="s">
+        <v>1084</v>
+      </c>
+      <c r="H98" t="s">
+        <v>49</v>
+      </c>
+      <c r="I98" t="s">
         <v>1085</v>
       </c>
-      <c r="H98" t="s">
-        <v>49</v>
-      </c>
-      <c r="I98" t="s">
+      <c r="J98" t="s">
         <v>1086</v>
-      </c>
-      <c r="J98" t="s">
-        <v>1087</v>
       </c>
       <c r="K98" t="s">
         <v>844</v>
       </c>
       <c r="L98" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M98" t="s">
         <v>53</v>
@@ -16995,13 +16998,13 @@
         <v>211</v>
       </c>
       <c r="R98" t="s">
+        <v>1087</v>
+      </c>
+      <c r="S98" t="s">
+        <v>49</v>
+      </c>
+      <c r="T98" t="s">
         <v>1088</v>
-      </c>
-      <c r="S98" t="s">
-        <v>49</v>
-      </c>
-      <c r="T98" t="s">
-        <v>1089</v>
       </c>
       <c r="U98" t="s">
         <v>57</v>
@@ -17013,19 +17016,19 @@
         <v>163</v>
       </c>
       <c r="X98" t="s">
+        <v>1089</v>
+      </c>
+      <c r="Y98" t="s">
+        <v>865</v>
+      </c>
+      <c r="Z98" t="s">
         <v>1090</v>
-      </c>
-      <c r="Y98" t="s">
-        <v>866</v>
-      </c>
-      <c r="Z98" t="s">
-        <v>1091</v>
       </c>
       <c r="AA98" t="s">
         <v>148</v>
       </c>
       <c r="AB98" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="AC98" t="s">
         <v>774</v>
@@ -17067,7 +17070,7 @@
         <v>49</v>
       </c>
       <c r="AP98" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="99" spans="1:42" x14ac:dyDescent="0.3">
@@ -17078,34 +17081,34 @@
         <v>43</v>
       </c>
       <c r="C99" t="s">
+        <v>904</v>
+      </c>
+      <c r="D99" t="s">
         <v>905</v>
       </c>
-      <c r="D99" t="s">
+      <c r="E99" t="s">
         <v>906</v>
-      </c>
-      <c r="E99" t="s">
-        <v>907</v>
       </c>
       <c r="F99" t="s">
         <v>89</v>
       </c>
       <c r="G99" t="s">
+        <v>907</v>
+      </c>
+      <c r="H99" t="s">
         <v>908</v>
       </c>
-      <c r="H99" t="s">
+      <c r="I99" t="s">
+        <v>908</v>
+      </c>
+      <c r="J99" t="s">
         <v>909</v>
       </c>
-      <c r="I99" t="s">
-        <v>909</v>
-      </c>
-      <c r="J99" t="s">
-        <v>910</v>
-      </c>
       <c r="K99" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L99" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M99" t="s">
         <v>53</v>
@@ -17123,13 +17126,13 @@
         <v>626</v>
       </c>
       <c r="R99" t="s">
+        <v>1093</v>
+      </c>
+      <c r="S99" t="s">
+        <v>49</v>
+      </c>
+      <c r="T99" t="s">
         <v>1094</v>
-      </c>
-      <c r="S99" t="s">
-        <v>49</v>
-      </c>
-      <c r="T99" t="s">
-        <v>1095</v>
       </c>
       <c r="U99" t="s">
         <v>57</v>
@@ -17141,19 +17144,19 @@
         <v>163</v>
       </c>
       <c r="X99" t="s">
+        <v>1095</v>
+      </c>
+      <c r="Y99" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z99" t="s">
         <v>1096</v>
-      </c>
-      <c r="Y99" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z99" t="s">
-        <v>1097</v>
       </c>
       <c r="AA99" t="s">
         <v>148</v>
       </c>
       <c r="AB99" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="AC99" t="s">
         <v>774</v>
@@ -17195,7 +17198,7 @@
         <v>49</v>
       </c>
       <c r="AP99" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="100" spans="1:42" x14ac:dyDescent="0.3">
@@ -17206,34 +17209,34 @@
         <v>43</v>
       </c>
       <c r="C100" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D100" t="s">
         <v>1100</v>
       </c>
-      <c r="D100" t="s">
+      <c r="E100" t="s">
         <v>1101</v>
-      </c>
-      <c r="E100" t="s">
-        <v>1102</v>
       </c>
       <c r="F100" t="s">
         <v>156</v>
       </c>
       <c r="G100" t="s">
+        <v>1102</v>
+      </c>
+      <c r="H100" t="s">
+        <v>49</v>
+      </c>
+      <c r="I100" t="s">
         <v>1103</v>
       </c>
-      <c r="H100" t="s">
-        <v>49</v>
-      </c>
-      <c r="I100" t="s">
+      <c r="J100" t="s">
         <v>1104</v>
       </c>
-      <c r="J100" t="s">
-        <v>1105</v>
-      </c>
       <c r="K100" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L100" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M100" t="s">
         <v>53</v>
@@ -17245,19 +17248,19 @@
         <v>139</v>
       </c>
       <c r="P100" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="Q100" t="s">
         <v>211</v>
       </c>
       <c r="R100" t="s">
+        <v>1106</v>
+      </c>
+      <c r="S100" t="s">
+        <v>49</v>
+      </c>
+      <c r="T100" t="s">
         <v>1107</v>
-      </c>
-      <c r="S100" t="s">
-        <v>49</v>
-      </c>
-      <c r="T100" t="s">
-        <v>1108</v>
       </c>
       <c r="U100" t="s">
         <v>57</v>
@@ -17269,19 +17272,19 @@
         <v>163</v>
       </c>
       <c r="X100" t="s">
+        <v>1108</v>
+      </c>
+      <c r="Y100" t="s">
+        <v>865</v>
+      </c>
+      <c r="Z100" t="s">
         <v>1109</v>
-      </c>
-      <c r="Y100" t="s">
-        <v>866</v>
-      </c>
-      <c r="Z100" t="s">
-        <v>1110</v>
       </c>
       <c r="AA100" t="s">
         <v>148</v>
       </c>
       <c r="AB100" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="AC100" t="s">
         <v>774</v>
@@ -17323,7 +17326,7 @@
         <v>49</v>
       </c>
       <c r="AP100" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="101" spans="1:42" x14ac:dyDescent="0.3">
@@ -17334,34 +17337,34 @@
         <v>43</v>
       </c>
       <c r="C101" t="s">
+        <v>1112</v>
+      </c>
+      <c r="D101" t="s">
         <v>1113</v>
       </c>
-      <c r="D101" t="s">
+      <c r="E101" t="s">
         <v>1114</v>
-      </c>
-      <c r="E101" t="s">
-        <v>1115</v>
       </c>
       <c r="F101" t="s">
         <v>156</v>
       </c>
       <c r="G101" t="s">
+        <v>1115</v>
+      </c>
+      <c r="H101" t="s">
         <v>1116</v>
       </c>
-      <c r="H101" t="s">
+      <c r="I101" t="s">
+        <v>1116</v>
+      </c>
+      <c r="J101" t="s">
         <v>1117</v>
-      </c>
-      <c r="I101" t="s">
-        <v>1117</v>
-      </c>
-      <c r="J101" t="s">
-        <v>1118</v>
       </c>
       <c r="K101" t="s">
         <v>844</v>
       </c>
       <c r="L101" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M101" t="s">
         <v>53</v>
@@ -17397,10 +17400,10 @@
         <v>163</v>
       </c>
       <c r="X101" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="Y101" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Z101" t="s">
         <v>161</v>
@@ -17409,7 +17412,7 @@
         <v>178</v>
       </c>
       <c r="AB101" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="AC101" t="s">
         <v>774</v>
@@ -17451,7 +17454,7 @@
         <v>49</v>
       </c>
       <c r="AP101" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="102" spans="1:42" x14ac:dyDescent="0.3">
@@ -17462,34 +17465,34 @@
         <v>43</v>
       </c>
       <c r="C102" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D102" t="s">
         <v>1122</v>
       </c>
-      <c r="D102" t="s">
+      <c r="E102" t="s">
         <v>1123</v>
-      </c>
-      <c r="E102" t="s">
-        <v>1124</v>
       </c>
       <c r="F102" t="s">
         <v>371</v>
       </c>
       <c r="G102" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H102" t="s">
         <v>1125</v>
       </c>
-      <c r="H102" t="s">
+      <c r="I102" t="s">
+        <v>1125</v>
+      </c>
+      <c r="J102" t="s">
         <v>1126</v>
-      </c>
-      <c r="I102" t="s">
-        <v>1126</v>
-      </c>
-      <c r="J102" t="s">
-        <v>1127</v>
       </c>
       <c r="K102" t="s">
         <v>817</v>
       </c>
       <c r="L102" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M102" t="s">
         <v>53</v>
@@ -17498,7 +17501,7 @@
         <v>54</v>
       </c>
       <c r="O102" t="s">
-        <v>854</v>
+        <v>55</v>
       </c>
       <c r="P102" t="s">
         <v>55</v>
@@ -17507,13 +17510,13 @@
         <v>76</v>
       </c>
       <c r="R102" t="s">
+        <v>1127</v>
+      </c>
+      <c r="S102" t="s">
+        <v>49</v>
+      </c>
+      <c r="T102" t="s">
         <v>1128</v>
-      </c>
-      <c r="S102" t="s">
-        <v>49</v>
-      </c>
-      <c r="T102" t="s">
-        <v>1129</v>
       </c>
       <c r="U102" t="s">
         <v>57</v>
@@ -17525,25 +17528,25 @@
         <v>79</v>
       </c>
       <c r="X102" t="s">
+        <v>1129</v>
+      </c>
+      <c r="Y102" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z102" t="s">
         <v>1130</v>
-      </c>
-      <c r="Y102" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z102" t="s">
-        <v>1131</v>
       </c>
       <c r="AA102" t="s">
         <v>226</v>
       </c>
       <c r="AB102" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="AC102" t="s">
         <v>774</v>
       </c>
       <c r="AD102" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="AE102" t="s">
         <v>456</v>
@@ -17579,7 +17582,7 @@
         <v>49</v>
       </c>
       <c r="AP102" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="103" spans="1:42" x14ac:dyDescent="0.3">
@@ -17590,34 +17593,34 @@
         <v>43</v>
       </c>
       <c r="C103" t="s">
+        <v>1133</v>
+      </c>
+      <c r="D103" t="s">
         <v>1134</v>
       </c>
-      <c r="D103" t="s">
+      <c r="E103" t="s">
         <v>1135</v>
-      </c>
-      <c r="E103" t="s">
-        <v>1136</v>
       </c>
       <c r="F103" t="s">
         <v>89</v>
       </c>
       <c r="G103" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H103" t="s">
+        <v>49</v>
+      </c>
+      <c r="I103" t="s">
         <v>1137</v>
       </c>
-      <c r="H103" t="s">
-        <v>49</v>
-      </c>
-      <c r="I103" t="s">
+      <c r="J103" t="s">
         <v>1138</v>
       </c>
-      <c r="J103" t="s">
-        <v>1139</v>
-      </c>
       <c r="K103" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L103" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M103" t="s">
         <v>53</v>
@@ -17626,10 +17629,10 @@
         <v>54</v>
       </c>
       <c r="O103" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="P103" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="Q103" t="s">
         <v>211</v>
@@ -17656,7 +17659,7 @@
         <v>538</v>
       </c>
       <c r="Y103" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Z103" t="s">
         <v>350</v>
@@ -17707,7 +17710,7 @@
         <v>49</v>
       </c>
       <c r="AP103" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="104" spans="1:42" x14ac:dyDescent="0.3">
@@ -17718,34 +17721,34 @@
         <v>43</v>
       </c>
       <c r="C104" t="s">
+        <v>1141</v>
+      </c>
+      <c r="D104" t="s">
         <v>1142</v>
       </c>
-      <c r="D104" t="s">
+      <c r="E104" t="s">
         <v>1143</v>
       </c>
-      <c r="E104" t="s">
+      <c r="F104" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G104" t="s">
         <v>1144</v>
       </c>
-      <c r="F104" t="s">
-        <v>1003</v>
-      </c>
-      <c r="G104" t="s">
+      <c r="H104" t="s">
+        <v>49</v>
+      </c>
+      <c r="I104" t="s">
         <v>1145</v>
       </c>
-      <c r="H104" t="s">
-        <v>49</v>
-      </c>
-      <c r="I104" t="s">
+      <c r="J104" t="s">
         <v>1146</v>
       </c>
-      <c r="J104" t="s">
-        <v>1147</v>
-      </c>
       <c r="K104" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L104" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M104" t="s">
         <v>53</v>
@@ -17757,7 +17760,7 @@
         <v>398</v>
       </c>
       <c r="P104" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="Q104" t="s">
         <v>57</v>
@@ -17784,13 +17787,13 @@
         <v>122</v>
       </c>
       <c r="Y104" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Z104" t="s">
         <v>49</v>
       </c>
       <c r="AA104" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="AB104" t="s">
         <v>122</v>
@@ -17835,7 +17838,7 @@
         <v>49</v>
       </c>
       <c r="AP104" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="105" spans="1:42" x14ac:dyDescent="0.3">
@@ -17846,34 +17849,34 @@
         <v>43</v>
       </c>
       <c r="C105" t="s">
+        <v>1141</v>
+      </c>
+      <c r="D105" t="s">
         <v>1142</v>
       </c>
-      <c r="D105" t="s">
+      <c r="E105" t="s">
         <v>1143</v>
       </c>
-      <c r="E105" t="s">
+      <c r="F105" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G105" t="s">
         <v>1144</v>
       </c>
-      <c r="F105" t="s">
-        <v>1003</v>
-      </c>
-      <c r="G105" t="s">
+      <c r="H105" t="s">
+        <v>49</v>
+      </c>
+      <c r="I105" t="s">
         <v>1145</v>
       </c>
-      <c r="H105" t="s">
-        <v>49</v>
-      </c>
-      <c r="I105" t="s">
+      <c r="J105" t="s">
         <v>1146</v>
       </c>
-      <c r="J105" t="s">
-        <v>1147</v>
-      </c>
       <c r="K105" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L105" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="M105" t="s">
         <v>53</v>
@@ -17885,7 +17888,7 @@
         <v>398</v>
       </c>
       <c r="P105" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="Q105" t="s">
         <v>57</v>
@@ -17912,13 +17915,13 @@
         <v>122</v>
       </c>
       <c r="Y105" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Z105" t="s">
         <v>49</v>
       </c>
       <c r="AA105" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="AB105" t="s">
         <v>122</v>
@@ -17963,7 +17966,7 @@
         <v>49</v>
       </c>
       <c r="AP105" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="106" spans="1:42" x14ac:dyDescent="0.3">
@@ -17974,34 +17977,34 @@
         <v>43</v>
       </c>
       <c r="C106" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D106" t="s">
         <v>1151</v>
       </c>
-      <c r="D106" t="s">
+      <c r="E106" t="s">
         <v>1152</v>
-      </c>
-      <c r="E106" t="s">
-        <v>1153</v>
       </c>
       <c r="F106" t="s">
         <v>172</v>
       </c>
       <c r="G106" t="s">
+        <v>1153</v>
+      </c>
+      <c r="H106" t="s">
+        <v>49</v>
+      </c>
+      <c r="I106" t="s">
         <v>1154</v>
       </c>
-      <c r="H106" t="s">
-        <v>49</v>
-      </c>
-      <c r="I106" t="s">
+      <c r="J106" t="s">
         <v>1155</v>
       </c>
-      <c r="J106" t="s">
-        <v>1156</v>
-      </c>
       <c r="K106" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L106" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M106" t="s">
         <v>53</v>
@@ -18034,22 +18037,22 @@
         <v>57</v>
       </c>
       <c r="W106" t="s">
+        <v>1156</v>
+      </c>
+      <c r="X106" t="s">
         <v>1157</v>
       </c>
-      <c r="X106" t="s">
+      <c r="Y106" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z106" t="s">
         <v>1158</v>
-      </c>
-      <c r="Y106" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z106" t="s">
-        <v>1159</v>
       </c>
       <c r="AA106" t="s">
         <v>569</v>
       </c>
       <c r="AB106" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="AC106" t="s">
         <v>774</v>
@@ -18091,7 +18094,7 @@
         <v>49</v>
       </c>
       <c r="AP106" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="107" spans="1:42" x14ac:dyDescent="0.3">
@@ -18102,34 +18105,34 @@
         <v>43</v>
       </c>
       <c r="C107" t="s">
+        <v>1161</v>
+      </c>
+      <c r="D107" t="s">
         <v>1162</v>
       </c>
-      <c r="D107" t="s">
+      <c r="E107" t="s">
         <v>1163</v>
-      </c>
-      <c r="E107" t="s">
-        <v>1164</v>
       </c>
       <c r="F107" t="s">
         <v>89</v>
       </c>
       <c r="G107" t="s">
+        <v>1164</v>
+      </c>
+      <c r="H107" t="s">
+        <v>49</v>
+      </c>
+      <c r="I107" t="s">
         <v>1165</v>
       </c>
-      <c r="H107" t="s">
-        <v>49</v>
-      </c>
-      <c r="I107" t="s">
+      <c r="J107" t="s">
         <v>1166</v>
-      </c>
-      <c r="J107" t="s">
-        <v>1167</v>
       </c>
       <c r="K107" t="s">
         <v>684</v>
       </c>
       <c r="L107" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M107" t="s">
         <v>53</v>
@@ -18168,7 +18171,7 @@
         <v>243</v>
       </c>
       <c r="Y107" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z107" t="s">
         <v>244</v>
@@ -18177,7 +18180,7 @@
         <v>178</v>
       </c>
       <c r="AB107" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="AC107" t="s">
         <v>774</v>
@@ -18219,7 +18222,7 @@
         <v>49</v>
       </c>
       <c r="AP107" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="108" spans="1:42" x14ac:dyDescent="0.3">
@@ -18230,34 +18233,34 @@
         <v>43</v>
       </c>
       <c r="C108" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D108" t="s">
         <v>1170</v>
       </c>
-      <c r="D108" t="s">
+      <c r="E108" t="s">
         <v>1171</v>
-      </c>
-      <c r="E108" t="s">
-        <v>1172</v>
       </c>
       <c r="F108" t="s">
         <v>235</v>
       </c>
       <c r="G108" t="s">
+        <v>1172</v>
+      </c>
+      <c r="H108" t="s">
+        <v>49</v>
+      </c>
+      <c r="I108" t="s">
         <v>1173</v>
       </c>
-      <c r="H108" t="s">
-        <v>49</v>
-      </c>
-      <c r="I108" t="s">
+      <c r="J108" t="s">
         <v>1174</v>
       </c>
-      <c r="J108" t="s">
-        <v>1175</v>
-      </c>
       <c r="K108" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L108" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M108" t="s">
         <v>53</v>
@@ -18293,19 +18296,19 @@
         <v>163</v>
       </c>
       <c r="X108" t="s">
+        <v>1175</v>
+      </c>
+      <c r="Y108" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z108" t="s">
         <v>1176</v>
-      </c>
-      <c r="Y108" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z108" t="s">
-        <v>1177</v>
       </c>
       <c r="AA108" t="s">
         <v>148</v>
       </c>
       <c r="AB108" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="AC108" t="s">
         <v>774</v>
@@ -18347,7 +18350,7 @@
         <v>49</v>
       </c>
       <c r="AP108" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="109" spans="1:42" x14ac:dyDescent="0.3">
@@ -18358,34 +18361,34 @@
         <v>43</v>
       </c>
       <c r="C109" t="s">
+        <v>1179</v>
+      </c>
+      <c r="D109" t="s">
         <v>1180</v>
       </c>
-      <c r="D109" t="s">
+      <c r="E109" t="s">
         <v>1181</v>
-      </c>
-      <c r="E109" t="s">
-        <v>1182</v>
       </c>
       <c r="F109" t="s">
         <v>827</v>
       </c>
       <c r="G109" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H109" t="s">
+        <v>1182</v>
+      </c>
+      <c r="I109" t="s">
         <v>1016</v>
       </c>
-      <c r="H109" t="s">
-        <v>1183</v>
-      </c>
-      <c r="I109" t="s">
+      <c r="J109" t="s">
         <v>1017</v>
-      </c>
-      <c r="J109" t="s">
-        <v>1018</v>
       </c>
       <c r="K109" t="s">
         <v>659</v>
       </c>
       <c r="L109" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M109" t="s">
         <v>53</v>
@@ -18397,7 +18400,7 @@
         <v>139</v>
       </c>
       <c r="P109" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="Q109" t="s">
         <v>76</v>
@@ -18424,7 +18427,7 @@
         <v>410</v>
       </c>
       <c r="Y109" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z109" t="s">
         <v>411</v>
@@ -18433,7 +18436,7 @@
         <v>148</v>
       </c>
       <c r="AB109" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="AC109" t="s">
         <v>774</v>
@@ -18475,7 +18478,7 @@
         <v>49</v>
       </c>
       <c r="AP109" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="110" spans="1:42" x14ac:dyDescent="0.3">
@@ -18486,34 +18489,34 @@
         <v>43</v>
       </c>
       <c r="C110" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D110" t="s">
         <v>1186</v>
       </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
         <v>1187</v>
-      </c>
-      <c r="E110" t="s">
-        <v>1188</v>
       </c>
       <c r="F110" t="s">
         <v>156</v>
       </c>
       <c r="G110" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H110" t="s">
+        <v>49</v>
+      </c>
+      <c r="I110" t="s">
         <v>1189</v>
       </c>
-      <c r="H110" t="s">
-        <v>49</v>
-      </c>
-      <c r="I110" t="s">
+      <c r="J110" t="s">
         <v>1190</v>
-      </c>
-      <c r="J110" t="s">
-        <v>1191</v>
       </c>
       <c r="K110" t="s">
         <v>422</v>
       </c>
       <c r="L110" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M110" t="s">
         <v>53</v>
@@ -18552,7 +18555,7 @@
         <v>580</v>
       </c>
       <c r="Y110" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z110" t="s">
         <v>581</v>
@@ -18561,7 +18564,7 @@
         <v>148</v>
       </c>
       <c r="AB110" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="AC110" t="s">
         <v>774</v>
@@ -18603,7 +18606,7 @@
         <v>49</v>
       </c>
       <c r="AP110" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="111" spans="1:42" x14ac:dyDescent="0.3">
@@ -18614,34 +18617,34 @@
         <v>43</v>
       </c>
       <c r="C111" t="s">
+        <v>1193</v>
+      </c>
+      <c r="D111" t="s">
         <v>1194</v>
       </c>
-      <c r="D111" t="s">
+      <c r="E111" t="s">
         <v>1195</v>
-      </c>
-      <c r="E111" t="s">
-        <v>1196</v>
       </c>
       <c r="F111" t="s">
         <v>235</v>
       </c>
       <c r="G111" t="s">
+        <v>1196</v>
+      </c>
+      <c r="H111" t="s">
+        <v>49</v>
+      </c>
+      <c r="I111" t="s">
         <v>1197</v>
       </c>
-      <c r="H111" t="s">
-        <v>49</v>
-      </c>
-      <c r="I111" t="s">
+      <c r="J111" t="s">
         <v>1198</v>
       </c>
-      <c r="J111" t="s">
-        <v>1199</v>
-      </c>
       <c r="K111" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L111" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M111" t="s">
         <v>53</v>
@@ -18659,13 +18662,13 @@
         <v>95</v>
       </c>
       <c r="R111" t="s">
+        <v>896</v>
+      </c>
+      <c r="S111" t="s">
+        <v>49</v>
+      </c>
+      <c r="T111" t="s">
         <v>897</v>
-      </c>
-      <c r="S111" t="s">
-        <v>49</v>
-      </c>
-      <c r="T111" t="s">
-        <v>898</v>
       </c>
       <c r="U111" t="s">
         <v>57</v>
@@ -18677,19 +18680,19 @@
         <v>163</v>
       </c>
       <c r="X111" t="s">
+        <v>1047</v>
+      </c>
+      <c r="Y111" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z111" t="s">
         <v>1048</v>
-      </c>
-      <c r="Y111" t="s">
-        <v>876</v>
-      </c>
-      <c r="Z111" t="s">
-        <v>1049</v>
       </c>
       <c r="AA111" t="s">
         <v>148</v>
       </c>
       <c r="AB111" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="AC111" t="s">
         <v>774</v>
@@ -18731,7 +18734,7 @@
         <v>49</v>
       </c>
       <c r="AP111" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="112" spans="1:42" x14ac:dyDescent="0.3">
@@ -18742,34 +18745,34 @@
         <v>43</v>
       </c>
       <c r="C112" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D112" t="s">
         <v>1202</v>
       </c>
-      <c r="D112" t="s">
+      <c r="E112" t="s">
         <v>1203</v>
-      </c>
-      <c r="E112" t="s">
-        <v>1204</v>
       </c>
       <c r="F112" t="s">
         <v>235</v>
       </c>
       <c r="G112" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="H112" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="I112" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="J112" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="K112" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="L112" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M112" t="s">
         <v>53</v>
@@ -18805,19 +18808,19 @@
         <v>163</v>
       </c>
       <c r="X112" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="Y112" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z112" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="AA112" t="s">
         <v>148</v>
       </c>
       <c r="AB112" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="AC112" t="s">
         <v>774</v>
@@ -18859,7 +18862,7 @@
         <v>49</v>
       </c>
       <c r="AP112" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="113" spans="1:42" x14ac:dyDescent="0.3">
@@ -18870,13 +18873,13 @@
         <v>43</v>
       </c>
       <c r="C113" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D113" t="s">
         <v>1208</v>
       </c>
-      <c r="D113" t="s">
+      <c r="E113" t="s">
         <v>1209</v>
-      </c>
-      <c r="E113" t="s">
-        <v>1210</v>
       </c>
       <c r="F113" t="s">
         <v>89</v>
@@ -18885,19 +18888,19 @@
         <v>347</v>
       </c>
       <c r="H113" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="I113" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="J113" t="s">
         <v>349</v>
       </c>
       <c r="K113" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="L113" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="M113" t="s">
         <v>53</v>
@@ -18936,7 +18939,7 @@
         <v>481</v>
       </c>
       <c r="Y113" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="Z113" t="s">
         <v>512</v>
@@ -18987,7 +18990,7 @@
         <v>49</v>
       </c>
       <c r="AP113" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar CONSULTA_VENTA_PF.xlsx — 01-04-2026, 4:50:41 p. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_PF.xlsx
+++ b/datos/CONSULTA_VENTA_PF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{1210F783-412B-4AE0-A961-DAE578DA2515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F600A4C-811C-4744-8DB3-39192154BA39}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{A4A385CD-814A-4900-A08A-CCE1FF4630CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C45C5448-2C25-4451-A0C2-DB0DCF75D88F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="ParamQuery Pro" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ParamQuery Pro'!$A$1:$AP$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ParamQuery Pro'!$A$1:$AP$115</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4746" uniqueCount="1213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4830" uniqueCount="1236">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -3646,6 +3646,51 @@
     <t>4172</t>
   </si>
   <si>
+    <t>17960337-3</t>
+  </si>
+  <si>
+    <t>LAGOS BELMAR CAMILA PATRICIA</t>
+  </si>
+  <si>
+    <t>22/10/1991</t>
+  </si>
+  <si>
+    <t>65 - Ñuñoa - Santiago -CP</t>
+  </si>
+  <si>
+    <t>947509045</t>
+  </si>
+  <si>
+    <t>gabrielaproteccionfamiliar@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>7800000</t>
+  </si>
+  <si>
+    <t>6554622</t>
+  </si>
+  <si>
+    <t>780000</t>
+  </si>
+  <si>
+    <t>01/04/2026</t>
+  </si>
+  <si>
+    <t>7020000</t>
+  </si>
+  <si>
+    <t>146250</t>
+  </si>
+  <si>
+    <t>SERVICIO FUNERARIO TESOROS DEL ALMA SIEMPRE JUNTOS</t>
+  </si>
+  <si>
+    <t>SIEMPRE JUNTOS</t>
+  </si>
+  <si>
+    <t>4174</t>
+  </si>
+  <si>
     <t>19570796-0</t>
   </si>
   <si>
@@ -3661,7 +3706,31 @@
     <t>4175</t>
   </si>
   <si>
-    <t>Rodolfo Santana</t>
+    <t>6197099-1</t>
+  </si>
+  <si>
+    <t>MONTERO PARRAGUEZ JUANA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>22/08/1953</t>
+  </si>
+  <si>
+    <t>2627 - Santiago - Santiago -CP</t>
+  </si>
+  <si>
+    <t>+56979649</t>
+  </si>
+  <si>
+    <t>Gefernandez@uc.cl; ; ; ;</t>
+  </si>
+  <si>
+    <t>Carlos Patricio Freitas Vega</t>
+  </si>
+  <si>
+    <t>4176</t>
+  </si>
+  <si>
+    <t>Rodoldo Santana</t>
   </si>
 </sst>
 </file>
@@ -4522,10 +4591,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP113"/>
+  <dimension ref="A1:AP115"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="41" width="8" customWidth="1"/>
+    <col min="1" max="14" width="8" customWidth="1"/>
+    <col min="15" max="15" width="13.109375" customWidth="1"/>
+    <col min="16" max="41" width="8" customWidth="1"/>
     <col min="42" max="42" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5469,7 +5540,7 @@
         <v>54</v>
       </c>
       <c r="O8" t="s">
-        <v>1212</v>
+        <v>1235</v>
       </c>
       <c r="P8" t="s">
         <v>140</v>
@@ -5597,7 +5668,7 @@
         <v>54</v>
       </c>
       <c r="O9" t="s">
-        <v>1212</v>
+        <v>1235</v>
       </c>
       <c r="P9" t="s">
         <v>140</v>
@@ -18882,19 +18953,19 @@
         <v>1209</v>
       </c>
       <c r="F113" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="G113" t="s">
-        <v>347</v>
+        <v>1210</v>
       </c>
       <c r="H113" t="s">
-        <v>1210</v>
+        <v>49</v>
       </c>
       <c r="I113" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="J113" t="s">
-        <v>349</v>
+        <v>1212</v>
       </c>
       <c r="K113" t="s">
         <v>875</v>
@@ -18909,22 +18980,22 @@
         <v>54</v>
       </c>
       <c r="O113" t="s">
-        <v>55</v>
+        <v>338</v>
       </c>
       <c r="P113" t="s">
-        <v>319</v>
+        <v>637</v>
       </c>
       <c r="Q113" t="s">
-        <v>76</v>
+        <v>142</v>
       </c>
       <c r="R113" t="s">
-        <v>482</v>
+        <v>1213</v>
       </c>
       <c r="S113" t="s">
         <v>49</v>
       </c>
       <c r="T113" t="s">
-        <v>511</v>
+        <v>1214</v>
       </c>
       <c r="U113" t="s">
         <v>57</v>
@@ -18933,31 +19004,31 @@
         <v>57</v>
       </c>
       <c r="W113" t="s">
-        <v>257</v>
+        <v>163</v>
       </c>
       <c r="X113" t="s">
-        <v>481</v>
+        <v>1215</v>
       </c>
       <c r="Y113" t="s">
-        <v>875</v>
+        <v>1216</v>
       </c>
       <c r="Z113" t="s">
-        <v>512</v>
+        <v>1217</v>
       </c>
       <c r="AA113" t="s">
-        <v>822</v>
+        <v>178</v>
       </c>
       <c r="AB113" t="s">
-        <v>719</v>
+        <v>1218</v>
       </c>
       <c r="AC113" t="s">
         <v>774</v>
       </c>
       <c r="AD113" t="s">
-        <v>515</v>
+        <v>1219</v>
       </c>
       <c r="AE113" t="s">
-        <v>311</v>
+        <v>1220</v>
       </c>
       <c r="AF113" t="s">
         <v>65</v>
@@ -18990,7 +19061,263 @@
         <v>49</v>
       </c>
       <c r="AP113" t="s">
-        <v>1211</v>
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="114" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>42</v>
+      </c>
+      <c r="B114" t="s">
+        <v>43</v>
+      </c>
+      <c r="C114" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D114" t="s">
+        <v>1223</v>
+      </c>
+      <c r="E114" t="s">
+        <v>1224</v>
+      </c>
+      <c r="F114" t="s">
+        <v>89</v>
+      </c>
+      <c r="G114" t="s">
+        <v>347</v>
+      </c>
+      <c r="H114" t="s">
+        <v>1225</v>
+      </c>
+      <c r="I114" t="s">
+        <v>1225</v>
+      </c>
+      <c r="J114" t="s">
+        <v>349</v>
+      </c>
+      <c r="K114" t="s">
+        <v>875</v>
+      </c>
+      <c r="L114" t="s">
+        <v>875</v>
+      </c>
+      <c r="M114" t="s">
+        <v>53</v>
+      </c>
+      <c r="N114" t="s">
+        <v>54</v>
+      </c>
+      <c r="O114" t="s">
+        <v>55</v>
+      </c>
+      <c r="P114" t="s">
+        <v>319</v>
+      </c>
+      <c r="Q114" t="s">
+        <v>76</v>
+      </c>
+      <c r="R114" t="s">
+        <v>482</v>
+      </c>
+      <c r="S114" t="s">
+        <v>49</v>
+      </c>
+      <c r="T114" t="s">
+        <v>511</v>
+      </c>
+      <c r="U114" t="s">
+        <v>57</v>
+      </c>
+      <c r="V114" t="s">
+        <v>57</v>
+      </c>
+      <c r="W114" t="s">
+        <v>257</v>
+      </c>
+      <c r="X114" t="s">
+        <v>481</v>
+      </c>
+      <c r="Y114" t="s">
+        <v>875</v>
+      </c>
+      <c r="Z114" t="s">
+        <v>512</v>
+      </c>
+      <c r="AA114" t="s">
+        <v>822</v>
+      </c>
+      <c r="AB114" t="s">
+        <v>719</v>
+      </c>
+      <c r="AC114" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD114" t="s">
+        <v>515</v>
+      </c>
+      <c r="AE114" t="s">
+        <v>311</v>
+      </c>
+      <c r="AF114" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG114" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH114" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI114" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ114" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK114" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL114" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM114" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN114" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO114" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP114" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="115" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>42</v>
+      </c>
+      <c r="B115" t="s">
+        <v>43</v>
+      </c>
+      <c r="C115" t="s">
+        <v>1227</v>
+      </c>
+      <c r="D115" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E115" t="s">
+        <v>1229</v>
+      </c>
+      <c r="F115" t="s">
+        <v>394</v>
+      </c>
+      <c r="G115" t="s">
+        <v>1230</v>
+      </c>
+      <c r="H115" t="s">
+        <v>49</v>
+      </c>
+      <c r="I115" t="s">
+        <v>1231</v>
+      </c>
+      <c r="J115" t="s">
+        <v>1232</v>
+      </c>
+      <c r="K115" t="s">
+        <v>875</v>
+      </c>
+      <c r="L115" t="s">
+        <v>875</v>
+      </c>
+      <c r="M115" t="s">
+        <v>53</v>
+      </c>
+      <c r="N115" t="s">
+        <v>54</v>
+      </c>
+      <c r="O115" t="s">
+        <v>139</v>
+      </c>
+      <c r="P115" t="s">
+        <v>1233</v>
+      </c>
+      <c r="Q115" t="s">
+        <v>211</v>
+      </c>
+      <c r="R115" t="s">
+        <v>241</v>
+      </c>
+      <c r="S115" t="s">
+        <v>49</v>
+      </c>
+      <c r="T115" t="s">
+        <v>242</v>
+      </c>
+      <c r="U115" t="s">
+        <v>57</v>
+      </c>
+      <c r="V115" t="s">
+        <v>57</v>
+      </c>
+      <c r="W115" t="s">
+        <v>163</v>
+      </c>
+      <c r="X115" t="s">
+        <v>243</v>
+      </c>
+      <c r="Y115" t="s">
+        <v>1216</v>
+      </c>
+      <c r="Z115" t="s">
+        <v>244</v>
+      </c>
+      <c r="AA115" t="s">
+        <v>148</v>
+      </c>
+      <c r="AB115" t="s">
+        <v>1056</v>
+      </c>
+      <c r="AC115" t="s">
+        <v>774</v>
+      </c>
+      <c r="AD115" t="s">
+        <v>125</v>
+      </c>
+      <c r="AE115" t="s">
+        <v>126</v>
+      </c>
+      <c r="AF115" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG115" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH115" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI115" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ115" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK115" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL115" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM115" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN115" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO115" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP115" t="s">
+        <v>1234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar CONSULTA_VENTA_PF.xlsx — 01-04-2026, 5:16:57 p. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_PF.xlsx
+++ b/datos/CONSULTA_VENTA_PF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{A4A385CD-814A-4900-A08A-CCE1FF4630CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61742208-E2D6-4C6B-9B60-A48DE7ABC7FF}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{A4A385CD-814A-4900-A08A-CCE1FF4630CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B8C6E16-31EE-4C6E-97AD-30298B14A285}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4769" uniqueCount="1210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4810" uniqueCount="1210">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -4136,9 +4136,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4519,7 +4518,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:AP115"/>
+  <dimension ref="A1:AP116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="14" width="8" customWidth="1"/>
@@ -4972,7 +4971,7 @@
       <c r="S4" t="s">
         <v>49</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4">
         <v>1428571</v>
       </c>
       <c r="U4" t="s">
@@ -5100,7 +5099,7 @@
       <c r="S5" t="s">
         <v>49</v>
       </c>
-      <c r="T5" s="1">
+      <c r="T5">
         <v>1134454</v>
       </c>
       <c r="U5" t="s">
@@ -5228,7 +5227,7 @@
       <c r="S6" t="s">
         <v>49</v>
       </c>
-      <c r="T6" s="1">
+      <c r="T6">
         <v>1436975</v>
       </c>
       <c r="U6" t="s">
@@ -5356,7 +5355,7 @@
       <c r="S7" t="s">
         <v>49</v>
       </c>
-      <c r="T7" s="1">
+      <c r="T7">
         <v>1436975</v>
       </c>
       <c r="U7" t="s">
@@ -5484,7 +5483,7 @@
       <c r="S8" t="s">
         <v>49</v>
       </c>
-      <c r="T8" s="1">
+      <c r="T8">
         <v>1428571</v>
       </c>
       <c r="U8" t="s">
@@ -5612,7 +5611,7 @@
       <c r="S9" t="s">
         <v>49</v>
       </c>
-      <c r="T9" s="1">
+      <c r="T9">
         <v>6680672</v>
       </c>
       <c r="U9" t="s">
@@ -5740,7 +5739,7 @@
       <c r="S10" t="s">
         <v>49</v>
       </c>
-      <c r="T10" s="1">
+      <c r="T10">
         <v>1210084</v>
       </c>
       <c r="U10" t="s">
@@ -5868,7 +5867,7 @@
       <c r="S11" t="s">
         <v>49</v>
       </c>
-      <c r="T11" s="1">
+      <c r="T11">
         <v>2689076</v>
       </c>
       <c r="U11" t="s">
@@ -5996,7 +5995,7 @@
       <c r="S12" t="s">
         <v>49</v>
       </c>
-      <c r="T12" s="1">
+      <c r="T12">
         <v>2394958</v>
       </c>
       <c r="U12" t="s">
@@ -6124,7 +6123,7 @@
       <c r="S13" t="s">
         <v>49</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13">
         <v>2100840</v>
       </c>
       <c r="U13" t="s">
@@ -6252,7 +6251,7 @@
       <c r="S14" t="s">
         <v>49</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14">
         <v>1109244</v>
       </c>
       <c r="U14" t="s">
@@ -6380,7 +6379,7 @@
       <c r="S15" t="s">
         <v>49</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15">
         <v>2155462</v>
       </c>
       <c r="U15" t="s">
@@ -6508,7 +6507,7 @@
       <c r="S16" t="s">
         <v>49</v>
       </c>
-      <c r="T16" s="1">
+      <c r="T16">
         <v>2605042</v>
       </c>
       <c r="U16" t="s">
@@ -6636,7 +6635,7 @@
       <c r="S17" t="s">
         <v>49</v>
       </c>
-      <c r="T17" s="1">
+      <c r="T17">
         <v>2268908</v>
       </c>
       <c r="U17" t="s">
@@ -6764,7 +6763,7 @@
       <c r="S18" t="s">
         <v>49</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18">
         <v>2647059</v>
       </c>
       <c r="U18" t="s">
@@ -6892,7 +6891,7 @@
       <c r="S19" t="s">
         <v>49</v>
       </c>
-      <c r="T19" s="1">
+      <c r="T19">
         <v>2899160</v>
       </c>
       <c r="U19" t="s">
@@ -7020,7 +7019,7 @@
       <c r="S20" t="s">
         <v>49</v>
       </c>
-      <c r="T20" s="1">
+      <c r="T20">
         <v>2352941</v>
       </c>
       <c r="U20" t="s">
@@ -7148,7 +7147,7 @@
       <c r="S21" t="s">
         <v>49</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21">
         <v>2142857</v>
       </c>
       <c r="U21" t="s">
@@ -7276,7 +7275,7 @@
       <c r="S22" t="s">
         <v>49</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22">
         <v>1575630</v>
       </c>
       <c r="U22" t="s">
@@ -7404,7 +7403,7 @@
       <c r="S23" t="s">
         <v>49</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23">
         <v>1361345</v>
       </c>
       <c r="U23" t="s">
@@ -7532,7 +7531,7 @@
       <c r="S24" t="s">
         <v>49</v>
       </c>
-      <c r="T24" s="1">
+      <c r="T24">
         <v>1796218</v>
       </c>
       <c r="U24" t="s">
@@ -7660,7 +7659,7 @@
       <c r="S25" t="s">
         <v>49</v>
       </c>
-      <c r="T25" s="1">
+      <c r="T25">
         <v>1796218</v>
       </c>
       <c r="U25" t="s">
@@ -7788,7 +7787,7 @@
       <c r="S26" t="s">
         <v>49</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26">
         <v>2857143</v>
       </c>
       <c r="U26" t="s">
@@ -7916,7 +7915,7 @@
       <c r="S27" t="s">
         <v>49</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27">
         <v>2857143</v>
       </c>
       <c r="U27" t="s">
@@ -8044,7 +8043,7 @@
       <c r="S28" t="s">
         <v>49</v>
       </c>
-      <c r="T28" s="1">
+      <c r="T28">
         <v>2394958</v>
       </c>
       <c r="U28" t="s">
@@ -8172,7 +8171,7 @@
       <c r="S29" t="s">
         <v>49</v>
       </c>
-      <c r="T29" s="1">
+      <c r="T29">
         <v>1361345</v>
       </c>
       <c r="U29" t="s">
@@ -8300,7 +8299,7 @@
       <c r="S30" t="s">
         <v>49</v>
       </c>
-      <c r="T30" s="1">
+      <c r="T30">
         <v>2226891</v>
       </c>
       <c r="U30" t="s">
@@ -8428,7 +8427,7 @@
       <c r="S31" t="s">
         <v>49</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31">
         <v>2226891</v>
       </c>
       <c r="U31" t="s">
@@ -8556,7 +8555,7 @@
       <c r="S32" t="s">
         <v>49</v>
       </c>
-      <c r="T32" s="1">
+      <c r="T32">
         <v>1210084</v>
       </c>
       <c r="U32" t="s">
@@ -8684,7 +8683,7 @@
       <c r="S33" t="s">
         <v>49</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33">
         <v>3697479</v>
       </c>
       <c r="U33" t="s">
@@ -8812,7 +8811,7 @@
       <c r="S34" t="s">
         <v>49</v>
       </c>
-      <c r="T34" s="1">
+      <c r="T34">
         <v>1848739</v>
       </c>
       <c r="U34" t="s">
@@ -8940,7 +8939,7 @@
       <c r="S35" t="s">
         <v>49</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35">
         <v>1680672</v>
       </c>
       <c r="U35" t="s">
@@ -9068,7 +9067,7 @@
       <c r="S36" t="s">
         <v>49</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36">
         <v>1680672</v>
       </c>
       <c r="U36" t="s">
@@ -9196,7 +9195,7 @@
       <c r="S37" t="s">
         <v>49</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37">
         <v>2823529</v>
       </c>
       <c r="U37" t="s">
@@ -9324,7 +9323,7 @@
       <c r="S38" t="s">
         <v>49</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38">
         <v>1512605</v>
       </c>
       <c r="U38" t="s">
@@ -9452,7 +9451,7 @@
       <c r="S39" t="s">
         <v>49</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39">
         <v>1558824</v>
       </c>
       <c r="U39" t="s">
@@ -9580,7 +9579,7 @@
       <c r="S40" t="s">
         <v>49</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40">
         <v>1512605</v>
       </c>
       <c r="U40" t="s">
@@ -9708,7 +9707,7 @@
       <c r="S41" t="s">
         <v>49</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41">
         <v>2521008</v>
       </c>
       <c r="U41" t="s">
@@ -9836,7 +9835,7 @@
       <c r="S42" t="s">
         <v>49</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42">
         <v>1882353</v>
       </c>
       <c r="U42" t="s">
@@ -9964,7 +9963,7 @@
       <c r="S43" t="s">
         <v>49</v>
       </c>
-      <c r="T43" s="1">
+      <c r="T43">
         <v>2004202</v>
       </c>
       <c r="U43" t="s">
@@ -10092,7 +10091,7 @@
       <c r="S44" t="s">
         <v>49</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44">
         <v>924370</v>
       </c>
       <c r="U44" t="s">
@@ -10220,7 +10219,7 @@
       <c r="S45" t="s">
         <v>49</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45">
         <v>1478992</v>
       </c>
       <c r="U45" t="s">
@@ -10348,7 +10347,7 @@
       <c r="S46" t="s">
         <v>49</v>
       </c>
-      <c r="T46" s="1">
+      <c r="T46">
         <v>1857143</v>
       </c>
       <c r="U46" t="s">
@@ -10476,7 +10475,7 @@
       <c r="S47" t="s">
         <v>49</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47">
         <v>1558824</v>
       </c>
       <c r="U47" t="s">
@@ -10604,7 +10603,7 @@
       <c r="S48" t="s">
         <v>49</v>
       </c>
-      <c r="T48" s="1">
+      <c r="T48">
         <v>2004202</v>
       </c>
       <c r="U48" t="s">
@@ -10732,7 +10731,7 @@
       <c r="S49" t="s">
         <v>49</v>
       </c>
-      <c r="T49" s="1">
+      <c r="T49">
         <v>1680672</v>
       </c>
       <c r="U49" t="s">
@@ -10860,7 +10859,7 @@
       <c r="S50" t="s">
         <v>49</v>
       </c>
-      <c r="T50" s="1">
+      <c r="T50">
         <v>1884454</v>
       </c>
       <c r="U50" t="s">
@@ -10988,7 +10987,7 @@
       <c r="S51" t="s">
         <v>49</v>
       </c>
-      <c r="T51" s="1">
+      <c r="T51">
         <v>4201681</v>
       </c>
       <c r="U51" t="s">
@@ -11116,7 +11115,7 @@
       <c r="S52" t="s">
         <v>49</v>
       </c>
-      <c r="T52" s="1">
+      <c r="T52">
         <v>2174370</v>
       </c>
       <c r="U52" t="s">
@@ -11244,7 +11243,7 @@
       <c r="S53" t="s">
         <v>49</v>
       </c>
-      <c r="T53" s="1">
+      <c r="T53">
         <v>2004202</v>
       </c>
       <c r="U53" t="s">
@@ -11372,7 +11371,7 @@
       <c r="S54" t="s">
         <v>49</v>
       </c>
-      <c r="T54" s="1">
+      <c r="T54">
         <v>1512605</v>
       </c>
       <c r="U54" t="s">
@@ -11500,7 +11499,7 @@
       <c r="S55" t="s">
         <v>49</v>
       </c>
-      <c r="T55" s="1">
+      <c r="T55">
         <v>1680672</v>
       </c>
       <c r="U55" t="s">
@@ -11628,7 +11627,7 @@
       <c r="S56" t="s">
         <v>49</v>
       </c>
-      <c r="T56" s="1">
+      <c r="T56">
         <v>1680672</v>
       </c>
       <c r="U56" t="s">
@@ -11756,7 +11755,7 @@
       <c r="S57" t="s">
         <v>49</v>
       </c>
-      <c r="T57" s="1">
+      <c r="T57">
         <v>2155462</v>
       </c>
       <c r="U57" t="s">
@@ -11884,7 +11883,7 @@
       <c r="S58" t="s">
         <v>49</v>
       </c>
-      <c r="T58" s="1">
+      <c r="T58">
         <v>1218487</v>
       </c>
       <c r="U58" t="s">
@@ -12012,7 +12011,7 @@
       <c r="S59" t="s">
         <v>49</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59">
         <v>2004202</v>
       </c>
       <c r="U59" t="s">
@@ -12140,7 +12139,7 @@
       <c r="S60" t="s">
         <v>49</v>
       </c>
-      <c r="T60" s="1">
+      <c r="T60">
         <v>1512605</v>
       </c>
       <c r="U60" t="s">
@@ -12268,7 +12267,7 @@
       <c r="S61" t="s">
         <v>49</v>
       </c>
-      <c r="T61" s="1">
+      <c r="T61">
         <v>1386555</v>
       </c>
       <c r="U61" t="s">
@@ -12396,7 +12395,7 @@
       <c r="S62" t="s">
         <v>49</v>
       </c>
-      <c r="T62" s="1">
+      <c r="T62">
         <v>1344538</v>
       </c>
       <c r="U62" t="s">
@@ -12524,7 +12523,7 @@
       <c r="S63" t="s">
         <v>49</v>
       </c>
-      <c r="T63" s="1">
+      <c r="T63">
         <v>1512605</v>
       </c>
       <c r="U63" t="s">
@@ -12652,7 +12651,7 @@
       <c r="S64" t="s">
         <v>49</v>
       </c>
-      <c r="T64" s="1">
+      <c r="T64">
         <v>1218487</v>
       </c>
       <c r="U64" t="s">
@@ -19248,6 +19247,134 @@
       </c>
       <c r="AP115" t="s">
         <v>1208</v>
+      </c>
+    </row>
+    <row r="116" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>42</v>
+      </c>
+      <c r="B116" t="s">
+        <v>43</v>
+      </c>
+      <c r="C116" t="s">
+        <v>730</v>
+      </c>
+      <c r="D116" t="s">
+        <v>731</v>
+      </c>
+      <c r="E116" t="s">
+        <v>732</v>
+      </c>
+      <c r="F116" t="s">
+        <v>168</v>
+      </c>
+      <c r="G116" t="s">
+        <v>680</v>
+      </c>
+      <c r="H116" t="s">
+        <v>49</v>
+      </c>
+      <c r="I116" t="s">
+        <v>733</v>
+      </c>
+      <c r="J116" t="s">
+        <v>734</v>
+      </c>
+      <c r="K116" t="s">
+        <v>660</v>
+      </c>
+      <c r="L116" t="s">
+        <v>691</v>
+      </c>
+      <c r="M116" t="s">
+        <v>53</v>
+      </c>
+      <c r="N116" t="s">
+        <v>54</v>
+      </c>
+      <c r="O116" t="s">
+        <v>55</v>
+      </c>
+      <c r="P116" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q116" t="s">
+        <v>57</v>
+      </c>
+      <c r="R116" t="s">
+        <v>683</v>
+      </c>
+      <c r="S116" t="s">
+        <v>49</v>
+      </c>
+      <c r="T116">
+        <v>10000000</v>
+      </c>
+      <c r="U116" t="s">
+        <v>57</v>
+      </c>
+      <c r="V116" t="s">
+        <v>57</v>
+      </c>
+      <c r="W116" t="s">
+        <v>60</v>
+      </c>
+      <c r="X116" t="s">
+        <v>683</v>
+      </c>
+      <c r="Y116" t="s">
+        <v>691</v>
+      </c>
+      <c r="Z116" t="s">
+        <v>49</v>
+      </c>
+      <c r="AA116" t="s">
+        <v>233</v>
+      </c>
+      <c r="AB116" t="s">
+        <v>683</v>
+      </c>
+      <c r="AC116" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD116" t="s">
+        <v>223</v>
+      </c>
+      <c r="AE116" t="s">
+        <v>109</v>
+      </c>
+      <c r="AF116" t="s">
+        <v>65</v>
+      </c>
+      <c r="AG116" t="s">
+        <v>65</v>
+      </c>
+      <c r="AH116" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI116" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ116" t="s">
+        <v>65</v>
+      </c>
+      <c r="AK116" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL116" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM116" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN116" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO116" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP116" t="s">
+        <v>735</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar CONSULTA_VENTA_PF.xlsx — 02-04-2026, 5:13:17 p. m.
</commit_message>
<xml_diff>
--- a/datos/CONSULTA_VENTA_PF.xlsx
+++ b/datos/CONSULTA_VENTA_PF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{A4A385CD-814A-4900-A08A-CCE1FF4630CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B8C6E16-31EE-4C6E-97AD-30298B14A285}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{A4A385CD-814A-4900-A08A-CCE1FF4630CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB9E3661-CAEE-4972-B70D-3F97082557C8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4810" uniqueCount="1210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4769" uniqueCount="1210">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -4196,10 +4196,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -4517,8 +4513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:AP116"/>
+  <dimension ref="A1:AP115"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="14" width="8" customWidth="1"/>
@@ -4657,7 +4652,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -4785,7 +4780,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -5169,7 +5164,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -5297,7 +5292,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -5425,7 +5420,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -5553,7 +5548,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="9" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -5681,7 +5676,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="10" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -5937,7 +5932,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="12" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -6065,7 +6060,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="13" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -6321,7 +6316,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="15" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -6449,7 +6444,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="16" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -6577,7 +6572,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="17" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -6705,7 +6700,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="18" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -6833,7 +6828,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="19" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -7089,7 +7084,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="21" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>42</v>
       </c>
@@ -7217,7 +7212,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="22" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -7345,7 +7340,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="23" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -7729,7 +7724,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="26" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>42</v>
       </c>
@@ -7857,7 +7852,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="27" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>42</v>
       </c>
@@ -7985,7 +7980,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="28" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -8113,7 +8108,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="29" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -8241,7 +8236,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="30" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -8369,7 +8364,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="31" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -8497,7 +8492,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="32" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -8625,7 +8620,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="33" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -8753,7 +8748,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="34" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -8881,7 +8876,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="35" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -9009,7 +9004,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="36" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -9137,7 +9132,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="37" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -9265,7 +9260,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="38" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -9393,7 +9388,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="39" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>42</v>
       </c>
@@ -9521,7 +9516,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="40" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>42</v>
       </c>
@@ -9649,7 +9644,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="41" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>42</v>
       </c>
@@ -9777,7 +9772,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="42" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>42</v>
       </c>
@@ -9905,7 +9900,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="43" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -10033,7 +10028,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="44" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>42</v>
       </c>
@@ -10161,7 +10156,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="45" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>42</v>
       </c>
@@ -10289,7 +10284,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="46" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>42</v>
       </c>
@@ -10417,7 +10412,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="47" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>42</v>
       </c>
@@ -10545,7 +10540,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="48" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>42</v>
       </c>
@@ -10673,7 +10668,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="49" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>42</v>
       </c>
@@ -10801,7 +10796,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="50" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>42</v>
       </c>
@@ -10929,7 +10924,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="51" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>42</v>
       </c>
@@ -11057,7 +11052,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="52" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>42</v>
       </c>
@@ -11313,7 +11308,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="54" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>42</v>
       </c>
@@ -11441,7 +11436,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="55" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>42</v>
       </c>
@@ -11569,7 +11564,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="56" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>42</v>
       </c>
@@ -11697,7 +11692,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="57" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>42</v>
       </c>
@@ -11953,7 +11948,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="59" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>42</v>
       </c>
@@ -12081,7 +12076,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="60" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>42</v>
       </c>
@@ -12209,7 +12204,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="61" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>42</v>
       </c>
@@ -12337,7 +12332,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="62" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>42</v>
       </c>
@@ -12465,7 +12460,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="63" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>42</v>
       </c>
@@ -12721,7 +12716,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="65" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>42</v>
       </c>
@@ -12849,7 +12844,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="66" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>42</v>
       </c>
@@ -12977,7 +12972,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="67" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>42</v>
       </c>
@@ -13105,7 +13100,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="68" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>42</v>
       </c>
@@ -13233,7 +13228,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="69" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>42</v>
       </c>
@@ -13361,7 +13356,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="70" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>42</v>
       </c>
@@ -13489,7 +13484,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="71" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>42</v>
       </c>
@@ -13617,7 +13612,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="72" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>42</v>
       </c>
@@ -13745,7 +13740,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="73" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>42</v>
       </c>
@@ -13873,7 +13868,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="74" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>42</v>
       </c>
@@ -14001,7 +13996,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="75" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>42</v>
       </c>
@@ -14129,7 +14124,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="76" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>42</v>
       </c>
@@ -14257,7 +14252,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="77" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>42</v>
       </c>
@@ -14385,7 +14380,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="78" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>42</v>
       </c>
@@ -14513,7 +14508,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="79" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>42</v>
       </c>
@@ -14641,7 +14636,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="80" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>42</v>
       </c>
@@ -14769,7 +14764,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="81" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>42</v>
       </c>
@@ -14897,7 +14892,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="82" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>42</v>
       </c>
@@ -15025,7 +15020,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="83" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>42</v>
       </c>
@@ -15153,7 +15148,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="84" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>42</v>
       </c>
@@ -15281,7 +15276,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="85" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>42</v>
       </c>
@@ -15409,7 +15404,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="86" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>42</v>
       </c>
@@ -15537,7 +15532,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="87" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>42</v>
       </c>
@@ -15665,7 +15660,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="88" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>42</v>
       </c>
@@ -15793,7 +15788,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="89" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>42</v>
       </c>
@@ -15921,7 +15916,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="90" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>42</v>
       </c>
@@ -16049,7 +16044,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="91" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>42</v>
       </c>
@@ -16177,7 +16172,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="92" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>42</v>
       </c>
@@ -16305,7 +16300,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="93" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>42</v>
       </c>
@@ -16433,7 +16428,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="94" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>42</v>
       </c>
@@ -16561,7 +16556,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="95" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>42</v>
       </c>
@@ -16689,7 +16684,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="96" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>42</v>
       </c>
@@ -16817,7 +16812,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="97" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>42</v>
       </c>
@@ -16945,7 +16940,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="98" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>42</v>
       </c>
@@ -17073,7 +17068,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="99" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>42</v>
       </c>
@@ -17201,7 +17196,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="100" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>42</v>
       </c>
@@ -17329,7 +17324,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="101" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>42</v>
       </c>
@@ -17457,7 +17452,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="102" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>42</v>
       </c>
@@ -17585,7 +17580,7 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="103" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>42</v>
       </c>
@@ -17713,7 +17708,7 @@
         <v>1114</v>
       </c>
     </row>
-    <row r="104" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>42</v>
       </c>
@@ -17841,7 +17836,7 @@
         <v>1122</v>
       </c>
     </row>
-    <row r="105" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>42</v>
       </c>
@@ -17969,7 +17964,7 @@
         <v>1123</v>
       </c>
     </row>
-    <row r="106" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>42</v>
       </c>
@@ -18097,7 +18092,7 @@
         <v>1134</v>
       </c>
     </row>
-    <row r="107" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>42</v>
       </c>
@@ -18225,7 +18220,7 @@
         <v>1142</v>
       </c>
     </row>
-    <row r="108" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>42</v>
       </c>
@@ -18353,7 +18348,7 @@
         <v>1152</v>
       </c>
     </row>
-    <row r="109" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>42</v>
       </c>
@@ -18481,7 +18476,7 @@
         <v>1158</v>
       </c>
     </row>
-    <row r="110" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>42</v>
       </c>
@@ -18609,7 +18604,7 @@
         <v>1166</v>
       </c>
     </row>
-    <row r="111" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>42</v>
       </c>
@@ -18737,7 +18732,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="112" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>42</v>
       </c>
@@ -18865,7 +18860,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="113" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>42</v>
       </c>
@@ -18993,7 +18988,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="114" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>42</v>
       </c>
@@ -19121,7 +19116,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="115" spans="1:42" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>42</v>
       </c>
@@ -19249,147 +19244,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="116" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>42</v>
-      </c>
-      <c r="B116" t="s">
-        <v>43</v>
-      </c>
-      <c r="C116" t="s">
-        <v>730</v>
-      </c>
-      <c r="D116" t="s">
-        <v>731</v>
-      </c>
-      <c r="E116" t="s">
-        <v>732</v>
-      </c>
-      <c r="F116" t="s">
-        <v>168</v>
-      </c>
-      <c r="G116" t="s">
-        <v>680</v>
-      </c>
-      <c r="H116" t="s">
-        <v>49</v>
-      </c>
-      <c r="I116" t="s">
-        <v>733</v>
-      </c>
-      <c r="J116" t="s">
-        <v>734</v>
-      </c>
-      <c r="K116" t="s">
-        <v>660</v>
-      </c>
-      <c r="L116" t="s">
-        <v>691</v>
-      </c>
-      <c r="M116" t="s">
-        <v>53</v>
-      </c>
-      <c r="N116" t="s">
-        <v>54</v>
-      </c>
-      <c r="O116" t="s">
-        <v>55</v>
-      </c>
-      <c r="P116" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q116" t="s">
-        <v>57</v>
-      </c>
-      <c r="R116" t="s">
-        <v>683</v>
-      </c>
-      <c r="S116" t="s">
-        <v>49</v>
-      </c>
-      <c r="T116">
-        <v>10000000</v>
-      </c>
-      <c r="U116" t="s">
-        <v>57</v>
-      </c>
-      <c r="V116" t="s">
-        <v>57</v>
-      </c>
-      <c r="W116" t="s">
-        <v>60</v>
-      </c>
-      <c r="X116" t="s">
-        <v>683</v>
-      </c>
-      <c r="Y116" t="s">
-        <v>691</v>
-      </c>
-      <c r="Z116" t="s">
-        <v>49</v>
-      </c>
-      <c r="AA116" t="s">
-        <v>233</v>
-      </c>
-      <c r="AB116" t="s">
-        <v>683</v>
-      </c>
-      <c r="AC116" t="s">
-        <v>62</v>
-      </c>
-      <c r="AD116" t="s">
-        <v>223</v>
-      </c>
-      <c r="AE116" t="s">
-        <v>109</v>
-      </c>
-      <c r="AF116" t="s">
-        <v>65</v>
-      </c>
-      <c r="AG116" t="s">
-        <v>65</v>
-      </c>
-      <c r="AH116" t="s">
-        <v>65</v>
-      </c>
-      <c r="AI116" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ116" t="s">
-        <v>65</v>
-      </c>
-      <c r="AK116" t="s">
-        <v>65</v>
-      </c>
-      <c r="AL116" t="s">
-        <v>49</v>
-      </c>
-      <c r="AM116" t="s">
-        <v>66</v>
-      </c>
-      <c r="AN116" t="s">
-        <v>49</v>
-      </c>
-      <c r="AO116" t="s">
-        <v>49</v>
-      </c>
-      <c r="AP116" t="s">
-        <v>735</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AP115" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="14">
-      <filters>
-        <filter val="WALTER FERRO"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="15">
-      <filters>
-        <filter val="ASDREYM CAROLINA GUILLEN VALDES"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>